<commit_message>
Add initial HTML structure and JavaScript for Product Costing module
- Created pc-price-reference.html, pc-produk.html, pc-simulasi.html with basic HTML structure.
- Implemented pc-shell.js for shared layout and menu functionality.
- Added pc.css for styling the Product Costing interface.
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="18.005" customWidth="1" style="1" min="1" max="1"/>
@@ -612,6 +612,40 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>Production Planning (eksternal, read-only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Master Material</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Data master material (Berat/Meter dll.) untuk costing dan unpack</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Engineering (first pass, belum dikonfirmasi klien)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Master rate, BOM, flow process, price reference, kurs dan simulasi costing/pricelist</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Accounting (first pass, belum dikonfirmasi klien)</t>
         </is>
       </c>
     </row>
@@ -833,12 +867,13 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Master Product (sesuai SPK); Baby Coil hasil Add Coil (bisa &gt;1); Qty; pilihan metode berat (Pilihan 1: Qty x Berat Standard/pcs, atau Pilihan 2: input Kg langsung); Berat Standard/pcs (database)</t>
+          <t>Master Product (sesuai SPK); Baby Coil hasil Add Coil (bisa &gt;1); Qty; pilihan metode berat (Pilihan 1: Qty x Berat Standard/pcs, atau Pilihan 2: input Kg langsung); Berat Standard/pcs (dihitung: Berat/Meter varian BOM × Panjang produk)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>FR-09: Admin Produksi menginput Detail Produksi untuk Finish Good KW 1 per baby coil yang sudah di-add (bisa &gt;1 baby coil per produk), dengan dua pilihan metode input berat: Pilihan 1 (Qty x Berat Standard/pcs dari database) atau Pilihan 2 (input Kg langsung, sistem hitung Berat/Pcs = Total Berat / Qty). Kedua pilihan menghasilkan %Selisih = (Berat/pcs - Berat Standard/pcs) / Berat Standard/pcs, dan sistem menampilkan popup notifikasi cek ulang bila selisih melebihi ± 0,7%.</t>
+          <t>FR-09: Admin Produksi menginput Detail Produksi untuk Finish Good KW 1 per baby coil yang sudah di-add (bisa &gt;1 baby coil per produk), dengan dua pilihan metode input berat: Pilihan 1 (Qty x Berat Standard/pcs dari database) atau Pilihan 2 (input Kg langsung, sistem hitung Berat/Pcs = Total Berat / Qty). Kedua pilihan menghasilkan %Selisih = (Berat/pcs - Berat Standard/pcs) / Berat Standard/pcs, dan sistem menampilkan popup notifikasi cek ulang bila selisih melebihi ± 0,7%.
+Diubah 2026-10-07: Berat Standard/pcs bukan kolom database produk, melainkan hasil perhitungan = Berat/Meter varian BOM yang dipilih × Panjang produk (FR-37, FR-46); nilainya tersimpan ke berat_standard pada item laporan.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1170,7 +1205,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="10.005" customWidth="1" style="1" min="1" max="1"/>
@@ -1296,7 +1331,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FR-10: Admin Produksi dapat mencatat Stok Bebas untuk sisa coil yang dijadikan produk di luar SPK (bukan hasil SPK yang sedang berjalan), dengan alur input yang identik dengan FR-09 (pilihan Master Product, baby coil sumber, dua pilihan input berat, %Selisih, popup toleransi).
+          <t>FR-10: Admin Produksi dapat mencatat Stok Bebas untuk sisa coil yang dijadikan produk di luar SPK (bukan hasil SPK yang sedang berjalan), dengan alur input yang identik dengan FR-09 (pilihan Master Product, baby coil sumber, dua pilihan input berat, %Selisih, popup toleransi). Berat Standard/pcs dihitung dari Berat/Meter varian BOM × Panjang produk (lihat FR-09, diubah 2026-10-07).
 Dipisah dari UC-04 (Input Jumlah FG KW1) karena tujuan aktor berbeda — mencatat produk di luar SPK, bukan hasil SPK yang berjalan — meski dilakukan dalam sesi Laporan Produksi yang sama.</t>
         </is>
       </c>
@@ -1393,6 +1428,479 @@
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>warehouse_stock, baby_coil</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>UC-N05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Kelola Master Produk</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Master Product</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Level 1 Product Type; Level 2 Product Category; Level 3 Product Jenis; Level 4 Product Master (nama produk); Lebar; Tebal; Panjang (meter)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>FR-37: Master Produk menyimpan hierarki 4 level (Level 1 Product Type, Level 2 Product Category, Level 3 Product Jenis, Level 4 Product Master/nama produk) dan Lebar (tetap per produk, karena satu lebar bisa memakai ketebalan material berbeda). Tebal dan Panjang (meter) tetap disimpan di Master Produk (keputusan user 2026-10-07, open question 3; menggantikan catatan sheet Ide E9–E11). Berat per Pcs tidak disimpan di produk: = Berat/Meter varian BOM × Panjang produk (FR-46). Contoh user: Produk 1 panjang 6 m; material A 1 kg/m → 6 kg, material B 1,3 kg/m → 7,8 kg.
+Sub-flow:
+1. Engineering membuka daftar Master Produk.
+2. Engineering menambah/mengubah/menghapus produk: mengisi hierarki 4 level, Lebar, Tebal, dan Panjang (meter).
+3. Sistem menyimpan dan menampilkan kembali daftar produk. (Berat per Pcs tidak diisi di sini — diturunkan dari Berat/Meter varian BOM × Panjang.)
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Open question 3 resolved: Tebal dan Panjang tetap ada di Master Produk; berat per pcs = Berat/Meter varian BOM × Panjang. Aktor ditetapkan user 2026-10-07 (open question 10).</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Produk (hierarki 4 level, Lebar, Tebal, Panjang) tersimpan dan tampil di daftar Master Produk</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>product_lvl_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>UC-N06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Kelola Master Material</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Master Material</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Metal Type; Slitted/Non Slit; Boron/Non Boron; Material Name; Width; Thickness; Berat/Meter (kg/m)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>FR-38: Master Material menyimpan Metal Type, Slitted/Non Slit, Boron/Non Boron, Material Name, Width, Thickness, dan Berat/Meter (kg/m). Berat/Meter ditambahkan ke master karena dibutuhkan untuk konversi biaya dari Rp/Kg ke Rp/meter (catatan sheet Simulasi Program, I10), dan dipakai per varian BOM untuk menghitung Berat per Pcs. Contoh baris di sheet menulis Width 914 untuk material "…-1219-…"; itu salah ketik, nilai yang benar 1219 (input/2026-10-07-product-costing-jawaban/).
+Sub-flow:
+1. Engineering membuka daftar Master Material.
+2. Engineering menambah/mengubah/menghapus material dengan mengisi atribut di atas, termasuk Berat/Meter.
+3. Sistem menyimpan dan menampilkan kembali daftar material.
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Open question 8 resolved: Width yang benar 1219 (salah ketik pada contoh). Aktor ditetapkan user 2026-10-07 (open question 10).</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Material (termasuk Berat/Meter) tersimpan dan tampil di daftar Master Material</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>UC-N07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Kelola Kurs</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Currency; Kurs</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>FR-39: Master Kurs menyimpan Currency, Kurs, Last Updated, dan Updated By. Kurs dipakai mengubah Price Reference dari USD ke Rupiah.
+Sub-flow:
+1. Accounting membuka daftar Kurs.
+2. Accounting menambah/mengubah/menghapus Currency dan nilai Kurs.
+3. Sistem mengisi Last Updated dan Updated By, lalu menampilkan kembali daftar.
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Kurs dipakai oleh UC-N08 untuk mengubah Price Reference USD ke Rupiah. Aktor Accounting sesuai kolom Updated By pada sumber.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Kurs tersimpan dengan Last Updated dan Updated By; tampil di daftar Kurs</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>master_kurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>UC-N08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Kelola Price Reference</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Material; Harga pembelian per bulan (USD/kg); Keputusan Pemakaian Price Reference per material (Harga Terakhir atau Rata-rata)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>FR-40: Price Reference per material: (a) History Pembelian — harga/unit (USD/kg) per bulan; (b) sistem menurunkan Harga Pembelian Terakhir (harga bulan terisi paling baru) dan Harga Pembelian Rata-rata (rata-rata bulan yang terisi); (c) per material, user memilih Keputusan Pemakaian Price Reference — "Harga Terakhir" atau rata-rata — dan pilihan itu dapat diubah; (d) Final Price Reference (USD) = harga sesuai pilihan; Final Price Reference (IDR/kg) = Final USD × Kurs.
+Sub-flow:
+1. Purchasing memilih material dan mengisi/mengubah History Pembelian (harga USD/kg per bulan).
+2. Sistem menurunkan Harga Pembelian Terakhir (bulan terisi paling baru) dan Harga Pembelian Rata-rata (rata-rata bulan terisi) dan menampilkannya.
+3. Purchasing memilih Keputusan Pemakaian Price Reference per material: 'Harga Terakhir' atau 'Rata-rata' (dapat diubah).
+4. Sistem menampilkan Final Price Reference (USD) sesuai pilihan dan Final Price Reference (IDR/kg) = Final USD × Kurs (master Kurs, UC-N07).
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. User menetapkan seluruh UC ini kepada Purchasing, termasuk pilihan 'Harga Terakhir' vs 'Rata-rata' per material (user 2026-10-07; open question 10).</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>History Pembelian, Harga Terakhir, Harga Rata-rata, Final Price Reference USD dan IDR/kg per material tersimpan dan tampil</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>history_purchase, price_reference_header, price_reference_detail, material, master_kurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>UC-N09</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Kelola BOM Produk</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Produk; Varian Thickness (dipilih dari Master Material); material per varian</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>FR-41: BOM Produk: satu produk punya satu atau lebih varian BOM, dibedakan oleh ketebalan material (Varian Thickness diambil dari Master Material). Setiap varian punya No. Uniq ID sendiri (mis. Type 001.1, Type 001.2), Latest Update, dan Update By; aksi View, Edit, Delete. Satu produk boleh memakai beberapa varian material sekaligus.
+Sub-flow:
+1. Engineering membuka daftar BOM per produk.
+2. Engineering menambah varian BOM untuk produk: memilih material/ketebalan dari Master Material (satu produk boleh memakai beberapa varian sekaligus).
+3. Sistem membuat No. Uniq ID per varian (mis. Type 001.1, Type 001.2) dan mengisi Latest Update dan Update By.
+4. Engineering dapat View, Edit, atau Delete varian.
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Aktor Engineering sesuai kolom Updated By BOM pada sumber.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>BOM produk dengan varian, No. Uniq ID, Latest Update, dan Update By tersimpan dan tampil di daftar BOM</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>bom_header, bom_detail, product_lvl_4, material</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>UC-N10</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Kelola Flow Process &amp; Cycletime</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Costcentre/Area; Process Name; Machine; Cycletime (menit per meter); Man Power (jumlah orang)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>FR-42: Flow Process &amp; Cycletime: per proses menyimpan Costcentre/Area, Process Name, Machine, Cycletime (menit per meter), Man Power (jumlah orang), dan Man Hour = Cycletime × Man Power ÷ 60 (jam per meter). Total Man Hour = jumlah Man Hour seluruh proses pada flow. Contoh sheet: Cutting Spandek, mesin 24 m/menit → cycletime 1 ÷ 24 = 0,0417 menit/meter, 1 man power → 0,000694 jam/meter. Flow dikunci per Product Category (Level 2), bukan per produk Level 4 (keputusan user 2026-10-07; open question 1).
+Sub-flow:
+1. Engineering membuka flow process (per Product Category / Level 2).
+2. Engineering menambah/mengubah/menghapus proses pada flow: mengisi Costcentre/Area, Process Name, Machine, Cycletime, dan Man Power.
+3. Sistem menghitung Man Hour per proses = Cycletime × Man Power ÷ 60 dan Total Man Hour flow, lalu menampilkannya.
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Kunci flow: Product Category (open question 1, resolved). Aktor ditetapkan user 2026-10-07 (open question 10).</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Flow process dengan Man Hour per proses dan Total Man Hour tersimpan dan tampil</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>flow_process_header, flow_process_detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>UC-N11</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Kelola Man Power Rate</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Komponen Salary Direct Man Power; komponen BPJS (nilai rupiah input manual); komponen Biaya Lain-Lain; Faktor Indirect Labor; jam kerja per bulan (parameter); periode (bulan)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>FR-43: Man Power Rate dihitung dari tiga kelompok komponen per bulan: Salary Direct Man Power (Gaji Pokok, Tunjangan Keluarga, Tunjangan Jabatan, THR, Cuti, Uang Makan, Transport), BPJS (Jaminan Kecelakaan Kerja 0,89%, Kematian 0,3%, Hari Tua 3,7%, Pensiun 2%, Kesehatan 4%) — nilai rupiah tiap komponen BPJS diinput manual (persentase hanya keterangan) — dan Biaya Lain-Lain (Seragam, Sepatu, Helm, Sarung Tangan, Masker — dihitung prorate per bulan). Lalu: Total Biaya Direct Labor/Bulan = jumlah tiga kelompok; Rate Direct Labor = pembulatan ke atas (Total ÷ jam kerja per bulan, parameter yang di contoh bernilai 173 jam; layar menampilkan keterangan konstanta yang dipakai); Rate Man Power (Rp/jam) = Rate Direct Labor × Faktor Indirect Labor. Contoh sheet: 6.551.982,55 → 37.873 → × 1,5 = 56.809,5 per jam. Komponen dapat ditambah/dihapus per kelompok (tombol Add/Delete di sheet).
+Sub-flow:
+1. Accounting membuka Man Power Rate per bulan.
+2. Accounting mengisi/mengubah komponen pada tiga kelompok (Salary Direct Man Power, BPJS, Biaya Lain-Lain) dan dapat menambah/menghapus komponen per kelompok (nilai rupiah BPJS diinput manual), serta mengisi Faktor Indirect Labor dan parameter jam kerja per bulan.
+3. Sistem menghitung Total Biaya Direct Labor/Bulan, Rate Direct Labor (dibulatkan ke atas, Total ÷ jam kerja per bulan), lalu menampilkan keterangan konstanta jam yang dipakai, dan Rate Man Power (Rp/jam), lalu menampilkannya.
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Perubahan rate tidak mengubah laporan produksi yang sudah dibuat (FR-49 / NFR-09). Open question 7 resolved: BPJS input manual; 173 jam menjadi parameter dengan keterangan ditampilkan. Aktor ditetapkan user 2026-10-07 (open question 10).</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Rate Man Power (Rp/jam) beserta rincian komponen tersimpan dan tampil</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>man_power_rate, man_power_rate_component</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>UC-N12</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Kelola Rate Bahan Pendukung Khusus &amp; FOH</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Product Category (atau Level 4); Rate Bahan Pendukung Khusus (Rp/meter); Rate FOH (Rp/meter)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>FR-44: Rate Bahan Pendukung Khusus dan Rate FOH disimpan per Product Category dalam Rp/meter (contoh sheet: BONDECK 150 dan 400 — "contoh saja"). Kunci rate adalah Product Category (Level 2), bukan Level 4 (keputusan user 2026-10-07; open question 1).
+Sub-flow:
+1. Accounting membuka daftar rate Bahan Pendukung Khusus &amp; FOH.
+2. Accounting menambah/mengubah/menghapus rate per Product Category: Rate Bahan Pendukung Khusus dan Rate FOH dalam Rp/meter.
+3. Sistem menyimpan dan menampilkan kembali daftar rate.
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Perubahan rate tidak mengubah laporan produksi yang sudah dibuat (FR-49 / NFR-09). Kunci rate: Product Category (open question 1, resolved). Aktor ditetapkan user 2026-10-07 (open question 10).</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Rate Bahan Pendukung Khusus dan Rate FOH (Rp/meter) per kunci produk tersimpan dan tampil</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>rate_bahan_pendukung_foh</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>UC-N13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Kelola General Rate</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Consumables (%); Scrap (%); Biaya Koordinasi (Rp/Kg); Other Cost (Sales &amp; Marketing, Transport, Finance &amp; Admin, Management Fee, Interest, Profit; masing-masing %); Negotiation Allowance (%)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>FR-45: General Rate (berlaku semua produk): Consumables (% × Material Cost), Scrap (% × Material Cost), Biaya Koordinasi (Rp/Kg × Berat/Meter), Other Cost — Sales &amp; Marketing, Transport, Finance &amp; Admin, Management Fee, Interest, Profit (masing-masing % × HPP) — dan Negotiation Allowance (% × Bottom Price). Setiap baris punya jenis/satuan sendiri di master: Biaya Koordinasi = Rp/Kg, baris lainnya persentase. Contoh nilai di sheet: Consumables 5%, Scrap 2%, Koordinasi Rp200/Kg, Profit 5%, Negotiation Allowance 5%, lima Other Cost lain kosong (= 0). ERD menyediakan 6 slot Other Cost dan satu Negotiation Allowance.
+Sub-flow:
+1. Accounting membuka General Rate.
+2. Accounting mengisi/mengubah nilai Consumables, Scrap, Biaya Koordinasi, enam Other Cost, dan Negotiation Allowance (berlaku untuk semua produk).
+3. Sistem menyimpan dan menampilkan kembali nilai rate.
+Keputusan user 2026-10-07: master data dibangun dan diisi lewat UI sistem ini. Perubahan rate tidak mengubah laporan produksi yang sudah dibuat (FR-49 / NFR-09). Open question 11 resolved: tiap baris punya satuan/jenis sendiri (Koordinasi Rp/Kg, lainnya persentase). Aktor ditetapkan user 2026-10-07 (open question 10).</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>General Rate tersimpan dan tampil (satuan per baris: % atau Rp/Kg)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>rate_generals</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>UC-N14</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Lihat Simulasi Costing &amp; Pricelist</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Accounting, Sales, Engineering</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Produk (dan varian BOM); Ukuran Produk (meter) diambil otomatis dari Panjang Master Produk</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>FR-46: Sistem menghitung, untuk setiap kombinasi Produk × varian BOM, dalam Rp/meter: Price Reference (Rp/Kg) = Final Price Reference IDR material varian tersebut (FR-40); Material Cost = Price Reference (Rp/Kg) × Berat/Meter material (FR-38); Man Power Cost = Total Man Hour (FR-42) × Rate Man Power (FR-43); Bahan Pendukung Khusus, FOH = rate FR-44; Consumables = % × Material Cost; Scrap = % × Material Cost; Biaya Koordinasi = Rp/Kg × Berat/Meter (FR-45); HPP = Material + Man Power + Bahan Pendukung + FOH + Consumables + Scrap + Koordinasi; Other Cost (6 komponen) = % × HPP; Bottom Price = HPP + seluruh Other Cost; Negotiation Allowance = % × Bottom Price; Price List/Meter = Bottom Price + Negotiation Allowance. Setiap nilai juga ditampilkan dalam Rp/Kg = nilai Rp/meter ÷ Berat/Meter. Berat per Pcs varian BOM = Berat/Meter material varian × Panjang produk (FR-37). Material Cost memakai Berat/Meter material utuh tanpa faktor lebar produk (dikonfirmasi user 2026-10-07, open question 2).
+FR-47: Output Simulasi Costing menampilkan satu baris per Produk × varian BOM (No. Uniq ID, Price Reference USD/Kg, Kurs, Rp/Kg, Berat/Meter, seluruh komponen FR-46 dalam Rp/meter dan Rp/Kg), ditambah Ukuran Produk (meter) yang diambil otomatis dari Panjang Master Produk (FR-37; keputusan user 2026-10-07), Pricelist Produk/Meter (= Ukuran × Price List/Meter) dan Pricelist Produk/Kg, sebagai pembanding terhadap "Pricelist HFG saat ini" (contoh 27.400 Rp/Meter; hanya contoh pembanding hasil hitung pricelist klien dengan konsep mock up, user 2026-10-07). Struktur yang sama dikonfirmasi ERD: Product Costing Header/Detail.
+Sub-flow:
+1. Aktor membuka layar Simulasi Costing; Ukuran Produk (meter) terisi otomatis dari Panjang Master Produk.
+2. Sistem menghitung untuk setiap kombinasi Produk × varian BOM seluruh komponen FR-46 (Rp/meter dan Rp/Kg) dari master: Price Reference, Berat/Meter, Man Hour, Rate Man Power, rate Bahan Pendukung/FOH, General Rate, dan Kurs.
+3. Sistem menampilkan satu baris per Produk × varian BOM: No. Uniq ID, Price Reference USD/Kg, Kurs, Rp/Kg, Berat/Meter, seluruh komponen FR-46, Pricelist Produk/Meter dan Pricelist Produk/Kg (pembanding 'Pricelist HFG saat ini').
+Tiga aktor (Accounting, Sales, Engineering) masing-masing memakai layar ini secara independen sebagai tampilan baca/simulasi (user menyatakan semuanya ikut memperkirakan harga dasar); tidak ada handoff di tengah alur sehingga tetap satu UC (admission test 1 dan 5). Open question 2 (Material Cost memakai Berat/Meter material utuh), 9 (Pricelist HFG saat ini = Rp/Meter, contoh), dan 5/6 (Scrap dari Rate Generals; jam laporan tidak dihitung) sudah resolved. Rumus tidak ditambah di luar FR-46.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Tabel simulasi: satu baris per Produk × varian BOM dengan seluruh komponen biaya (Rp/meter dan Rp/Kg), Price List/Meter, serta Pricelist Produk/Meter dan /Kg</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>product_costing_header, product_costing_detail, material_cost, man_power_cost, bom_header, bom_detail, price_reference_header, flow_process_header, man_power_rate, rate_bahan_pendukung_foh, rate_generals, master_kurs, product_lvl_4</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1915,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="28.005" customWidth="1" style="1" min="1" max="1"/>
@@ -1506,12 +2014,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Unpack</t>
+          <t>Master Material</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Staf Gudang (master data, first pass)</t>
+          <t>Engineering (master data, first pass)</t>
         </is>
       </c>
       <c r="D5" s="3" t="b">
@@ -1611,7 +2119,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Admin Produksi (master data, first pass)</t>
+          <t>Engineering (master data, first pass)</t>
         </is>
       </c>
       <c r="D10" s="3" t="b">
@@ -1835,6 +2343,326 @@
         </is>
       </c>
       <c r="D21" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>master_kurs</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>history_purchase</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>price_reference_header</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>price_reference_detail</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>bom_header</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>bom_detail</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>flow_process_header</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>flow_process_detail</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>man_power_rate</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>rate_bahan_pendukung_foh</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>rate_generals</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>product_costing_header</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>product_costing_detail</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>material_cost</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>man_power_cost</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>man_power_rate_component</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D37" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(specs): perubahan rate Negotiation Allowance (Extra Margin) perlu approval GM
Sumber: BPM To Be Sales D01 (input) dan keputusan user 2026-10-21. Sales Manager mengajukan rate
baru per Product Category, GM Approve/Reject; rate aktif berubah hanya setelah Approved, Reject
kembali ke Sales Manager; Pricelist yang sudah diajukan tidak berubah (snapshot).
- fr-nfr: FR-67 baru, FR-55 direvisi, open question 20-24 (alasan Reject wajib diasumsikan).
- ERD: entitas rate_negotiation_allowance_request.
- workbook: UC-12 direvisi (Sales Manager), UC-16 baru (GM), PG-16 direvisi, PG-23 baru.
- vocabulary: Extra Margin; intake input/2026-10-21-sales-extra-margin-approval.
Persetujuan diskon Quotation, SO, SPM di luar scope Product Costing (modul Sales).

Refs FEAT-05 (tracker lokal; no issue di tracker eksternal)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -1263,12 +1263,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Tetapkan Rate Negotiation Allowance (Extra Margin) per Product Category</t>
+          <t>Ajukan Perubahan Rate Negotiation Allowance (Extra Margin) per Product Category</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1278,22 +1278,22 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Product Category; Rate Negotiation Allowance (Extra Margin, %)</t>
+          <t>Product Category; Rate Negotiation Allowance (Extra Margin, %) yang diajukan</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>FR-55 (user 2026-10-19). 1) Sales membuka daftar Rate Negotiation Allowance. 2) Sales menambah/mengubah/menghapus rate (%) per Product Category. 3) Sistem menyimpan, mengisi Latest Update dan Updated By, lalu menampilkan kembali daftar. Rate dipakai UC-13: Price List = Bottom Price + (Rate × Bottom Price); bukan lagi bagian Rate Generals. Dikerjakan berkala sesuai kebijakan. (Rev.1 UC-10; BPMN D05: 'Penetapan Rate Negotiation Allowance (Extra Margin)', lane Sales.)</t>
+          <t>FR-55 (direvisi 2026-10-21), FR-67. Prasyarat: produk sudah ada di Product Catalog (BPMN To Be Sales D01). 1) Sales Manager menilai "Perlu perubahan margin?" (acuan penilaian customer baru: toko sewa/sendiri, lama berdiri, armada, asset, jumlah cabang; tidak diotomasi). 2) Bila perlu, Sales Manager membuka halaman Negotiation Allowance dan mengajukan rate Extra Margin (%) baru untuk satu Product Category (angka ≥ 0, titik sebagai desimal; diasumsikan satu pengajuan per kategori, OQ 22). 3) Sistem menyimpan pengajuan berstatus Menunggu Approval GM beserta pengaju dan waktu; rate aktif TIDAK berubah, sehingga Simulasi, Pricelist, dan Katalog tetap memakai rate aktif. 4) Bila GM menolak (UC-16), pengajuan berstatus Rejected dengan alasan; Sales Manager memperbaiki lalu mengajukan ulang (pengajuan baru). Rate aktif dipakai UC-13: Price List = Bottom Price + (Rate × Bottom Price). Persetujuan diskon pada Quotation (&lt;5% Sales langsung, 5–10% Sales Manager, &gt;10% GM) di luar scope Product Costing. (Rev.1 UC-10, direvisi oleh BPMN To Be Sales D01 dan keputusan user 2026-10-21: perubahan rate perlu approval GM; BPMN D05: "Penetapan Rate Negotiation Allowance (Extra Margin)".)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Rate Negotiation Allowance per Product Category tersimpan, siap dipakai untuk generate Pricelist</t>
+          <t>Pengajuan perubahan rate berstatus Menunggu Approval GM tersimpan; rate aktif tidak berubah sampai disetujui GM (UC-16)</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>rate_negotiation_allowance</t>
+          <t>rate_negotiation_allowance_request, rate_negotiation_allowance</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>FR-47, FR-57, FR-58. Prasyarat: hasil costing sampai Bottom Price (UC-N14) dan UC-12 tersedia. 1) Sales memilih Produk (dan varian BOM) dan menerima Bottom Price dari hasil costing. 2) Sistem menghitung Price List = Bottom Price + (Rate Negotiation Allowance kategori × Bottom Price), Rp/Meter dan Rp/Kg, serta Pricelist Produk/Meter (= Ukuran Produk × Price List/Meter) dan Pricelist Produk/Kg sebagai pembanding terhadap Pricelist HFG saat ini (contoh 27.400 Rp/Meter, hanya contoh). 3) Sistem menghasilkan Report Costing Detail/Produk. 4) Sales menyusun Draft Pricelist per Produk × varian BOM (status Draft) dan mengirimnya ke Management (Menunggu Approval). Bila Management menolak (UC-14), Sales menghitung ulang dengan alasan Reject terlihat lalu mengajukan lagi. (Rev.1 UC-16 dan UC-17; BPMN D05: User task 'Pengajuan Approval Pricelist', service task 'Perhitungan Price List' dan dokumen 'Report Costing Detail/Product' dilipat.) Revisi 2026-10-20 (FR-59): Draft Pricelist boleh disimpan, tetapi tidak boleh diajukan ke Management selama ada baris yang datanya belum lengkap (rate, Price Reference, Faktor Indirect Labor, dst.); sistem menyebut kekurangan dan menu untuk mengisinya.</t>
+          <t>FR-47, FR-57, FR-58. Prasyarat: hasil costing sampai Bottom Price (UC-N14) dan rate Negotiation Allowance aktif tersedia (rate berubah hanya setelah pengajuan UC-12 disetujui GM di UC-16). 1) Sales memilih Produk (dan varian BOM) dan menerima Bottom Price dari hasil costing. 2) Sistem menghitung Price List = Bottom Price + (Rate Negotiation Allowance kategori × Bottom Price), Rp/Meter dan Rp/Kg, serta Pricelist Produk/Meter (= Ukuran Produk × Price List/Meter) dan Pricelist Produk/Kg sebagai pembanding terhadap Pricelist HFG saat ini (contoh 27.400 Rp/Meter, hanya contoh). 3) Sistem menghasilkan Report Costing Detail/Produk. 4) Sales menyusun Draft Pricelist per Produk × varian BOM (status Draft) dan mengirimnya ke Management (Menunggu Approval). Bila Management menolak (UC-14), Sales menghitung ulang dengan alasan Reject terlihat lalu mengajukan lagi. (Rev.1 UC-16 dan UC-17; BPMN D05: User task 'Pengajuan Approval Pricelist', service task 'Perhitungan Price List' dan dokumen 'Report Costing Detail/Product' dilipat.) Revisi 2026-10-20 (FR-59): Draft Pricelist boleh disimpan, tetapi tidak boleh diajukan ke Management selama ada baris yang datanya belum lengkap (rate, Price Reference, Faktor Indirect Labor, dst.); sistem menyebut kekurangan dan menu untuk mengisinya.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1443,7 +1443,53 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
+    <row r="17" ht="224" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>UC-16</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Setujui / Tolak Perubahan Rate Extra Margin</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Pengajuan perubahan rate Negotiation Allowance yang Menunggu Approval GM; keputusan Approve atau Reject; alasan Reject (wajib; diasumsikan, OQ 20)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>FR-67. Prasyarat: pengajuan berstatus Menunggu Approval GM (UC-12). 1) GM membuka antrean pengajuan perubahan rate Extra Margin. 2) GM membandingkan rate aktif dengan rate yang diajukan per Product Category, lalu memutuskan Approve atau Reject (alasan Reject wajib; diasumsikan, mohon konfirmasi). 3) Approve: sistem memperbarui rate aktif (rate_negotiation_allowance, latest_update, updated_by) dan menyimpan status Approved, decided_by, decided_at; rate baru dipakai Simulasi, Pricelist baru, dan Katalog berikutnya, sedangkan Pricelist yang sudah diajukan tidak berubah (snapshot, FR-58). 4) Reject: sistem menyimpan status Rejected, decided_by, decided_at, reject_reason; rate aktif tidak berubah; Sales Manager memperbaiki lalu mengajukan ulang (UC-12). Status pengajuan hanya Menunggu Approval GM, Approved, Rejected. (BPMN To Be Sales D01: gateway "Approval Extra Margin" di lane GM, Approved → Buat Quotation, Reject → "Update dan Ajukan Rate Extra Margin baru"; dijadikan UC karena keputusannya dibuat manusia.)</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Pengajuan Approved (rate aktif diperbarui) atau Rejected dengan alasan (kembali ke Sales Manager, UC-12)</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>rate_negotiation_allowance_request, rate_negotiation_allowance</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>PG-23</t>
+        </is>
+      </c>
+    </row>
     <row r="18"/>
     <row r="19"/>
     <row r="20"/>
@@ -1517,7 +1563,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -2380,34 +2426,948 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D129"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="28" customWidth="1" style="1" min="1" max="1"/>
+    <col width="16" customWidth="1" style="1" min="2" max="2"/>
+    <col width="8" customWidth="1" style="4" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Entity yang dibutuhkan</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Modul</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>ERD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>tr_unpack_coil_header</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Unpack</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>warehouse_pack</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Unpack</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>baby_coil</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Unpack</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Master Material</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Engineering (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>gudang_produksi_2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Gudang Produksi 2</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Staf Gudang (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>laporan_ketidaksesuaian_material</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Report Produksi</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>material_coil</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Report Produksi</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>PPIC</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>production_report_items</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Report Produksi</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Admin Produksi</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>product_lvl_4</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Master Product</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Engineering (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>production_report_scraps</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Report Produksi</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Admin Produksi</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>production_reports</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Report Produksi</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Admin Produksi</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>stok_gudang_wip</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Report Produksi</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Admin Produksi</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="98" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>production_plan</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Production Plan (Eksternal)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Production Planning (eksternal, read-only)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="98" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>asset</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Master Asset</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Staf Produksi (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="98" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>employee</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Master Employee</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Admin Produksi (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>jurnal_produksi</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Report HPP</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>gl_interface</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Report HPP</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>rate_negotiation_allowance</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>pricelist_header</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>pricelist_detail</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>product_costing_detail</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>product_catalog_header</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>product_catalog_detail</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" ht="84" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>gudang_material_hold</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Gudang Produksi 2</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Staf Gudang (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>production_report_materials</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Report Produksi</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Admin Produksi</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" ht="84" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>warehouse_stock</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Gudang Produksi 2</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Staf Gudang (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>master_kurs</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>history_purchase</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>price_reference_header</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>price_reference_detail</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>bom_header</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>bom_detail</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" ht="84" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>master_standard_material</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Master Material</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Engineering (master data, first pass)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>flow_process_header</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>flow_process_detail</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>man_power_rate</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Costing</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>man_power_rate_component</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Costing</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>rate_borongan_helper</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Costing</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>rate_bahan_pendukung_foh</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Costing</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>rate_generals</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Costing</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>product_costing_header</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>material_cost</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>man_power_cost</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>faktor_indirect_labor</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Costing</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>rate_negotiation_allowance_request</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
     <row r="47"/>
     <row r="48"/>
     <row r="49"/>
@@ -2441,928 +3401,56 @@
     <row r="77"/>
     <row r="78"/>
     <row r="79"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D45"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="28" customWidth="1" style="1" min="1" max="1"/>
-    <col width="16" customWidth="1" style="1" min="2" max="2"/>
-    <col width="8" customWidth="1" style="4" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Entity yang dibutuhkan</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Modul</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>ERD</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>tr_unpack_coil_header</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Unpack</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Operator</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>warehouse_pack</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Unpack</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Operator</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>baby_coil</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Unpack</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Operator</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" ht="84" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>material</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Master Material</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Engineering (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" ht="84" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>gudang_produksi_2</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Gudang Produksi 2</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Staf Gudang (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>laporan_ketidaksesuaian_material</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Report Produksi</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Operator</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>material_coil</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Report Produksi</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>PPIC</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>production_report_items</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Report Produksi</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Admin Produksi</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" ht="84" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>product_lvl_4</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Master Product</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Engineering (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>production_report_scraps</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Report Produksi</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Admin Produksi</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>production_reports</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Report Produksi</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Admin Produksi</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>stok_gudang_wip</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Report Produksi</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Admin Produksi</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="98" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>production_plan</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Production Plan (Eksternal)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Production Planning (eksternal, read-only)</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="98" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>asset</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Master Asset</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Staf Produksi (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" ht="98" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>employee</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Master Employee</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Admin Produksi (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>jurnal_produksi</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Report HPP</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Accounting</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>gl_interface</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Report HPP</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Accounting</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>rate_negotiation_allowance</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>pricelist_header</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>pricelist_detail</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>product_costing_detail</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Accounting</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>product_catalog_header</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>product_catalog_detail</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" ht="84" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>gudang_material_hold</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Gudang Produksi 2</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Staf Gudang (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>production_report_materials</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Report Produksi</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Admin Produksi</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" ht="84" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>warehouse_stock</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Gudang Produksi 2</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Staf Gudang (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>master_kurs</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>history_purchase</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Purchasing</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>price_reference_header</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>price_reference_detail</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>bom_header</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>bom_detail</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" ht="84" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>master_standard_material</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Master Material</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Engineering (master data, first pass)</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>flow_process_header</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>flow_process_detail</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>man_power_rate</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Costing</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>man_power_rate_component</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Costing</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>rate_borongan_helper</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Costing</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>rate_bahan_pendukung_foh</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Costing</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>rate_generals</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Costing</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>product_costing_header</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Accounting</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>material_cost</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Accounting</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>man_power_cost</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Accounting</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>faktor_indirect_labor</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>Product Costing</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Costing</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4330,7 +4418,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Sales menetapkan Rate Negotiation Allowance (%) per Product Category.</t>
+          <t>Sales Manager mengajukan perubahan Rate Negotiation Allowance (Extra Margin, %) per Product Category; rate aktif tidak berubah sampai disetujui GM (UC-16).</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -4340,7 +4428,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Sales: K</t>
+          <t>Sales Manager: K · GM: L</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -4350,7 +4438,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>usulan: aktor Sales, jadi halaman terpisah dari General Rate (Costing).</t>
+          <t>usulan: aktor Sales Manager (BPMN Sales D01), jadi halaman terpisah dari General Rate (Costing). Menampilkan rate aktif dan status pengajuan.</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -4701,7 +4789,63 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>PG-23</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Approval Extra Margin</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>/rate_negotiation_allowance/approval</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Halaman CI3 (antrean keputusan)</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>GM menyetujui atau menolak pengajuan perubahan Rate Negotiation Allowance (Extra Margin); Reject wajib beralasan (diasumsikan).</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>UC-16</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>GM: S · Sales Manager: L (alasan Reject)</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>usulan: antrean keputusan aktor lain (GM), halaman terpisah dari PG-16 dan dari Approval Pricelist (PG-19, Management); Area Rate karena objeknya rate master, bukan pricelist.</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>ui-mockup/pc-approval-extra-margin.html</t>
+        </is>
+      </c>
+    </row>
     <row r="25"/>
     <row r="26"/>
     <row r="27"/>

</xml_diff>

<commit_message>
docs(specs): dashboard notifikasi perubahan Bottom Price (FEAT-09, diusulkan)
Permintaan user 2026-10-21: alert ke Sales bila Bottom Price berubah, agar Sales menilai harga jual
dengan Rate Extra Margin lama dan memutuskan mengajukan rate baru (alur FR-67) atau tidak perlu diubah.
- fr-nfr: FR-68..FR-70, NFR-16, open question 25-33. Dikonfirmasi user: ambang sekecil apa pun,
  pembanding harga = Price List Product Catalog terakhir, peninjau semua Sales, kanal hanya
  dashboard, tanpa batas waktu tinjau. OQ 33: konsistensi pengaju Extra Margin dengan BPMN.
- ERD: entitas bottom_price_notification (diusulkan); workbook: UC-N18, PG-24; vocabulary;
  intake input/2026-10-21-bottom-price-change-notification; tracker FEAT-09 (open).

Refs FEAT-09 (tracker lokal; no issue di tracker eksternal)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1490,68 +1490,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1563,7 +1501,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -2426,6 +2364,53 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="409.5" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>UC-N18</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Tinjau Perubahan Bottom Price</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Notifikasi perubahan Bottom Price (per Produk × varian BOM, dikelompokkan per Product Category); keputusan "Ajukan Rate Extra Margin Baru" atau "Tidak Perlu Diubah"; catatan (opsional)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>FR-68, FR-69, FR-70, NFR-16 (diusulkan; ambang, pembanding harga, peninjau, dan kanal sudah dikonfirmasi user 2026-10-21 — OQ 25, 27, 28; sisanya diasumsikan, mohon konfirmasi OQ 26, 29–33). 1) Sistem membandingkan Bottom Price (Rp/Meter dan Rp/Kg) tiap Produk × varian BOM dengan baseline setiap kali costing dihitung; bila berbeda (naik atau turun, apa pun penyebabnya) sistem membuat notifikasi berstatus Belum Ditinjau (langkah otomatis, tanpa aktor). 2) Sales (Staf Sales atau Sales Manager) membuka dashboard notifikasi; notifikasi dikelompokkan per Product Category dan jumlah yang belum ditinjau tampil sebagai lencana di menu. 3) Sales membandingkan Bottom Price lama dan baru, selisih (Rp dan %), komponen yang berubah, Rate Extra Margin aktif, harga jual saat ini terhadap Price List baru bila rate lama dipertahankan. 4) Sales memilih: a) Ajukan Rate Extra Margin Baru: membuka pengajuan UC-12 untuk Product Category itu, lalu GM memutuskan di UC-16 (FR-67); status Diajukan Extra Margin Baru dan terhubung ke pengajuan; b) Tidak Perlu Diubah (catatan opsional): status Tidak Perlu Diubah. 5) Kedua keputusan mencatat peninjau, waktu, dan catatan, ditulis ke log, dan menggeser baseline ke Bottom Price baru. Sistem tidak mengubah rate, Pricelist, atau Katalog secara otomatis. Semua Sales dapat meninjau; kanal hanya dashboard (tanpa email/WhatsApp) dan tanpa batas waktu tinjau; ambang: perubahan sekecil apa pun (≥ Rp0,01). Di luar scope: persetujuan diskon Quotation. (Permintaan user 2026-10-21; terkait BPMN To Be Sales D01, gateway "Perlu Perubahan Margin?".)</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Notifikasi tertinjau: status Diajukan Extra Margin Baru (terhubung ke pengajuan UC-12) atau Tidak Perlu Diubah, dengan peninjau, waktu, dan catatan</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>bottom_price_notification, rate_negotiation_allowance, rate_negotiation_allowance_request, product_costing_detail</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>PG-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2437,7 +2422,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="28" customWidth="1" style="1" min="1" max="1"/>
@@ -3368,89 +3353,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>bottom_price_notification</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3462,7 +3384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4846,71 +4768,63 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>PG-24</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Hasil dan Pricelist</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard Notifikasi Bottom Price</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>/bottom_price_notification</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Halaman CI3 (daftar + modal Report Costing Detail)</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Menampilkan notifikasi bila Bottom Price Produk × varian BOM berubah (Bottom Price lama → baru, selisih, Rate Extra Margin aktif, harga jual saat ini vs Price List baru) agar Sales memutuskan Ajukan Rate Extra Margin Baru atau Tidak Perlu Diubah.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>UC-N18</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Sales: K (Staf Sales dan Sales Manager)</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>menu Hasil &amp; Pricelist; lencana jumlah notifikasi Belum Ditinjau di menu. Fitur diusulkan (FR-68–FR-70, NFR-16); rincian diasumsikan, open question 26, 29–33 (25, 27, 28 terjawab 2026-10-21). Path usulan.</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>baru (usulan); ui-mockup/pc-notifikasi-bottom-price.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(specs): konfirmasi user untuk notifikasi Bottom Price (OQ 25-33 terjawab)
Baseline = Bottom Price saat terakhir ditinjau; deteksi tiap costing dihitung ulang; satu keputusan per
notifikasi dan pengajuan per kategori; produk/BOM baru tidak memicu notifikasi; "Tidak Perlu Diubah"
cukup dengan catatan opsional. Pengajuan rate Extra Margin hanya Sales Manager (FR-67 tetap); semua
Sales dapat meninjau; hak akses diatur per pengguna di program. FR-68..70, UC-N18, PG-24 dan
catatan mockup disesuaikan.

Refs FEAT-09 (tracker lokal; no issue di tracker eksternal)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -2392,7 +2392,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>FR-68, FR-69, FR-70, NFR-16 (diusulkan; ambang, pembanding harga, peninjau, dan kanal sudah dikonfirmasi user 2026-10-21 — OQ 25, 27, 28; sisanya diasumsikan, mohon konfirmasi OQ 26, 29–33). 1) Sistem membandingkan Bottom Price (Rp/Meter dan Rp/Kg) tiap Produk × varian BOM dengan baseline setiap kali costing dihitung; bila berbeda (naik atau turun, apa pun penyebabnya) sistem membuat notifikasi berstatus Belum Ditinjau (langkah otomatis, tanpa aktor). 2) Sales (Staf Sales atau Sales Manager) membuka dashboard notifikasi; notifikasi dikelompokkan per Product Category dan jumlah yang belum ditinjau tampil sebagai lencana di menu. 3) Sales membandingkan Bottom Price lama dan baru, selisih (Rp dan %), komponen yang berubah, Rate Extra Margin aktif, harga jual saat ini terhadap Price List baru bila rate lama dipertahankan. 4) Sales memilih: a) Ajukan Rate Extra Margin Baru: membuka pengajuan UC-12 untuk Product Category itu, lalu GM memutuskan di UC-16 (FR-67); status Diajukan Extra Margin Baru dan terhubung ke pengajuan; b) Tidak Perlu Diubah (catatan opsional): status Tidak Perlu Diubah. 5) Kedua keputusan mencatat peninjau, waktu, dan catatan, ditulis ke log, dan menggeser baseline ke Bottom Price baru. Sistem tidak mengubah rate, Pricelist, atau Katalog secara otomatis. Semua Sales dapat meninjau; kanal hanya dashboard (tanpa email/WhatsApp) dan tanpa batas waktu tinjau; ambang: perubahan sekecil apa pun (≥ Rp0,01). Di luar scope: persetujuan diskon Quotation. (Permintaan user 2026-10-21; terkait BPMN To Be Sales D01, gateway "Perlu Perubahan Margin?".)</t>
+          <t>FR-68, FR-69, FR-70, NFR-16 (diusulkan; seluruh rincian dikonfirmasi user 2026-10-21 — OQ 25–33). 1) Sistem membandingkan Bottom Price (Rp/Meter dan Rp/Kg) tiap Produk × varian BOM dengan baseline setiap kali costing dihitung; bila berbeda (naik atau turun, apa pun penyebabnya) sistem membuat notifikasi berstatus Belum Ditinjau (langkah otomatis, tanpa aktor). 2) Sales (Staf Sales atau Sales Manager) membuka dashboard notifikasi; notifikasi dikelompokkan per Product Category dan jumlah yang belum ditinjau tampil sebagai lencana di menu. 3) Sales membandingkan Bottom Price lama dan baru, selisih (Rp dan %), komponen yang berubah, Rate Extra Margin aktif, harga jual saat ini terhadap Price List baru bila rate lama dipertahankan. 4) Sales memilih: a) Ajukan Rate Extra Margin Baru (hanya Sales Manager; hak akses diatur per pengguna di program): membuka pengajuan UC-12 untuk Product Category itu, lalu GM memutuskan di UC-16 (FR-67); status Diajukan Extra Margin Baru dan terhubung ke pengajuan; b) Tidak Perlu Diubah (catatan opsional): status Tidak Perlu Diubah. 5) Kedua keputusan mencatat peninjau, waktu, dan catatan, ditulis ke log, dan menggeser baseline ke Bottom Price baru. Sistem tidak mengubah rate, Pricelist, atau Katalog secara otomatis. Semua Sales dapat meninjau; kanal hanya dashboard (tanpa email/WhatsApp) dan tanpa batas waktu tinjau; ambang: perubahan sekecil apa pun (≥ Rp0,01). Di luar scope: persetujuan diskon Quotation. (Permintaan user 2026-10-21; terkait BPMN To Be Sales D01, gateway "Perlu Perubahan Margin?".)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Sales: K (Staf Sales dan Sales Manager)</t>
+          <t>Sales: K (lihat dan Tidak Perlu Diubah; Staf Sales dan Sales Manager) · Sales Manager: K (Ajukan Rate Extra Margin Baru; hak akses per pengguna di program)</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist; lencana jumlah notifikasi Belum Ditinjau di menu. Fitur diusulkan (FR-68–FR-70, NFR-16); rincian diasumsikan, open question 26, 29–33 (25, 27, 28 terjawab 2026-10-21). Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist; lencana jumlah notifikasi Belum Ditinjau di menu. Fitur diusulkan (FR-68–FR-70, NFR-16); rincian diasumsikan, open question 25–33 terjawab 2026-10-21. Path usulan.</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(specs): History Costing, History Price List, dan nama produk di Pricelist/Katalog (FEAT-10, diusulkan)
Permintaan user 2026-10-21: perubahan rate yang memengaruhi Bottom Price disimpan di History
Costing, perubahan Pricelist di History Price List; menu Pricelist dan Product Catalog menampilkan
nama produk, bukan nomor pricelist di depan.
- fr-nfr: FR-71..FR-73, NFR-17 (riwayat hanya baca), open question 34-42 (diasumsikan); FR-47
  dan FR-58 diberi catatan revisi tampilan.
- ERD: history_costing dan history_pricelist (diusulkan); workbook: UC-N19, UC-N20, PG-25, PG-26,
  catatan PG-18/PG-20; vocabulary; intake input/2026-10-21-history-costing-pricelist; tracker FEAT-10.

Refs FEAT-10 (tracker lokal; no issue di tracker eksternal)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -1330,7 +1330,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>FR-47, FR-57, FR-58. Prasyarat: hasil costing sampai Bottom Price (UC-N14) dan rate Negotiation Allowance aktif tersedia (rate berubah hanya setelah pengajuan UC-12 disetujui GM di UC-16). 1) Sales memilih Produk (dan varian BOM) dan menerima Bottom Price dari hasil costing. 2) Sistem menghitung Price List = Bottom Price + (Rate Negotiation Allowance kategori × Bottom Price), Rp/Meter dan Rp/Kg, serta Pricelist Produk/Meter (= Ukuran Produk × Price List/Meter) dan Pricelist Produk/Kg sebagai pembanding terhadap Pricelist HFG saat ini (contoh 27.400 Rp/Meter, hanya contoh). 3) Sistem menghasilkan Report Costing Detail/Produk. 4) Sales menyusun Draft Pricelist per Produk × varian BOM (status Draft) dan mengirimnya ke Management (Menunggu Approval). Bila Management menolak (UC-14), Sales menghitung ulang dengan alasan Reject terlihat lalu mengajukan lagi. (Rev.1 UC-16 dan UC-17; BPMN D05: User task 'Pengajuan Approval Pricelist', service task 'Perhitungan Price List' dan dokumen 'Report Costing Detail/Product' dilipat.) Revisi 2026-10-20 (FR-59): Draft Pricelist boleh disimpan, tetapi tidak boleh diajukan ke Management selama ada baris yang datanya belum lengkap (rate, Price Reference, Faktor Indirect Labor, dst.); sistem menyebut kekurangan dan menu untuk mengisinya.</t>
+          <t>FR-47, FR-57, FR-58. Prasyarat: hasil costing sampai Bottom Price (UC-N14) dan rate Negotiation Allowance aktif tersedia (rate berubah hanya setelah pengajuan UC-12 disetujui GM di UC-16). 1) Sales memilih Produk (dan varian BOM) dan menerima Bottom Price dari hasil costing. 2) Sistem menghitung Price List = Bottom Price + (Rate Negotiation Allowance kategori × Bottom Price), Rp/Meter dan Rp/Kg, serta Pricelist Produk/Meter (= Ukuran Produk × Price List/Meter) dan Pricelist Produk/Kg sebagai pembanding terhadap Pricelist HFG saat ini (contoh 27.400 Rp/Meter, hanya contoh). 3) Sistem menghasilkan Report Costing Detail/Produk. 4) Sales menyusun Draft Pricelist per Produk × varian BOM (status Draft) dan mengirimnya ke Management (Menunggu Approval). Bila Management menolak (UC-14), Sales menghitung ulang dengan alasan Reject terlihat lalu mengajukan lagi. (Rev.1 UC-16 dan UC-17; BPMN D05: User task 'Pengajuan Approval Pricelist', service task 'Perhitungan Price List' dan dokumen 'Report Costing Detail/Product' dilipat.) Revisi 2026-10-20 (FR-59): Draft Pricelist boleh disimpan, tetapi tidak boleh diajukan ke Management selama ada baris yang datanya belum lengkap (rate, Price Reference, Faktor Indirect Labor, dst.); sistem menyebut kekurangan dan menu untuk mengisinya. Tampilan daftar (revisi 2026-10-21, FR-73): nama produk (dengan varian/Uniq ID) di depan; nomor Pricelist/katalog menjadi kolom sekunder.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>FR-58. Prasyarat: pricelist Approved (UC-14). 1) Sales memilih Pricelist yang sudah Approved dan merilis Product Catalog. 2) Sistem menyimpan snapshot harga yang disetujui per Produk × varian BOM beserta released_by dan released_at (product_catalog_header/detail). 3) Product Catalog diteruskan ke proses Sales (di luar alur ini). Hanya pricelist Approved yang boleh dirilis; satu pricelist Approved boleh dirilis berkali-kali dan setiap rilis membuat Product Catalog (snapshot) baru (user 2026-10-20). (Rev.1 UC-18; BPMN D05 menggambarnya dengan ikon roda gigi, tetapi Use Case Rev.1 menyebut Sales yang merilis.)</t>
+          <t>FR-58. Prasyarat: pricelist Approved (UC-14). 1) Sales memilih Pricelist yang sudah Approved dan merilis Product Catalog. 2) Sistem menyimpan snapshot harga yang disetujui per Produk × varian BOM beserta released_by dan released_at (product_catalog_header/detail). 3) Product Catalog diteruskan ke proses Sales (di luar alur ini). Hanya pricelist Approved yang boleh dirilis; satu pricelist Approved boleh dirilis berkali-kali dan setiap rilis membuat Product Catalog (snapshot) baru (user 2026-10-20). (Rev.1 UC-18; BPMN D05 menggambarnya dengan ikon roda gigi, tetapi Use Case Rev.1 menyebut Sales yang merilis.) Tampilan daftar (revisi 2026-10-21, FR-73): nama produk (dengan varian/Uniq ID) di depan; nomor Pricelist/katalog menjadi kolom sekunder.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -2411,6 +2411,158 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="409.5" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>UC-N19</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Lihat History Costing</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Costing / Accounting / Sales / Management</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Filter: produk, Product Category, periode, sumber perubahan; pilihan catatan riwayat untuk melihat detail snapshot</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>FR-71, NFR-17 (diusulkan; rincian diasumsikan, mohon konfirmasi OQ 34–42). 1) Setiap kali perubahan master, rate, atau input costing membuat Bottom Price suatu Produk × varian BOM berubah, sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor): waktu, pengguna yang mengubah, sumber perubahan (master/rate yang diubah, nilai lama → baru), Bottom Price lama → baru (Rp/Meter dan Rp/Kg), snapshot komponen costing lama dan baru, dan Rate Extra Margin aktif. 2) Pengguna membuka halaman History Costing. 3) Pengguna menyaring menurut produk, Product Category, periode, dan sumber perubahan. 4) Pengguna membuka detail untuk melihat snapshot komponen lama dan baru. Riwayat hanya baca (tidak dapat diubah atau dihapus), dan terpisah dari Notifikasi Bottom Price (UC-N18): notifikasi untuk Sales meninjau, riwayat untuk audit. (Permintaan user 2026-10-21.)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Daftar riwayat perubahan Bottom Price dengan detail snapshot komponen lama dan baru</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>history_costing, product_costing_detail</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>PG-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="409.5" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>UC-N20</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Lihat History Price List</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Costing / Accounting / Sales / Management</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Filter: produk, Product Category, periode, kejadian; pilihan catatan riwayat untuk melihat detail</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>FR-72, NFR-17 (diusulkan; rincian diasumsikan, mohon konfirmasi OQ 34–42; terhubung ke FR-58 dan FR-67). 1) Setiap kejadian pada Pricelist disimpan per Produk × varian BOM (langkah otomatis, tanpa aktor): Diajukan, Disetujui (Approved), Ditolak (Rejected, beserta alasan), Dihitung Ulang (kembali ke Draft), atau Dirilis ke Product Catalog; dengan nomor Pricelist, status, waktu, pengguna, Price List lama → baru (Rp/Meter dan Rp/Kg), Bottom Price dan Rate Extra Margin saat itu, serta catatan atau alasan. 2) Pengguna membuka halaman History Price List. 3) Pengguna menyaring menurut produk, Product Category, periode, dan kejadian. 4) Pengguna melihat perubahan Price List lama → baru. Riwayat hanya baca (tidak dapat diubah atau dihapus). (Permintaan user 2026-10-21.)</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Daftar riwayat kejadian Pricelist per Produk × varian BOM dengan Price List lama dan baru</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>history_pricelist, pricelist_header, pricelist_detail, product_catalog_header</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>PG-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2422,7 +2574,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="28" customWidth="1" style="1" min="1" max="1"/>
@@ -3373,6 +3525,196 @@
         <v>1</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>history_costing</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>history_pricelist</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Product Costing</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3384,7 +3726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4474,7 +4816,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>usulan.</t>
+          <t>usulan. Revisi tampilan 2026-10-21 (FR-73): nama produk (dengan varian/Uniq ID) tampil di depan pada daftar; nomor Pricelist/katalog menjadi kolom sekunder.</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -4588,7 +4930,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>usulan.</t>
+          <t>usulan. Revisi tampilan 2026-10-21 (FR-73): nama produk (dengan varian/Uniq ID) tampil di depan pada daftar; nomor Pricelist/katalog menjadi kolom sekunder.</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -4825,6 +5167,212 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>PG-25</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Hasil dan Pricelist</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>History Costing</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>/history_costing</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Halaman CI3 (daftar + modal detail snapshot)</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Menampilkan riwayat perubahan Bottom Price per Produk × varian BOM (sumber perubahan, nilai lama → baru, snapshot komponen) untuk audit; hanya baca.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>UC-N19</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Costing, Accounting, Sales, Management: L</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-71, NFR-17); rincian diasumsikan, open question 34–42. Path usulan.</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>baru (usulan); ui-mockup/pc-history-costing.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>PG-26</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Hasil dan Pricelist</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>History Price List</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>/history_pricelist</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Halaman CI3 (daftar + modal detail)</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Menampilkan riwayat kejadian Pricelist (Diajukan, Disetujui, Ditolak, Dihitung Ulang, Dirilis) per Produk × varian BOM dengan Price List lama → baru; hanya baca.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>UC-N20</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Costing, Accounting, Sales, Management: L</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-72, NFR-17); rincian diasumsikan, open question 34–42. Path usulan.</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>baru (usulan); ui-mockup/pc-history-pricelist.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(specs): jawaban user untuk History Costing dan History Price List (OQ 34-40 terjawab)
- History Costing: dicatat bila costing diperbarui dan hasilnya berubah; persetujuan Extra Margin
  tidak dicatat.
- History Price List: hanya saat Pricelist Disetujui; Draft tidak dicatat.
- Masa simpan 1 tahun lalu dipindahkan ke backup data; akses oleh pengguna yang diberi hak akses;
  ekspor Excel; pencatatan lewat Activity Log (write_log).
- Open question baru 43-47 (Update Costing eksplisit, rilis katalog, akses backup, sumber data
  logs vs tabel khusus, hak akses lihat/ekspor). UC-N19/N20, PG-25/26 disesuaikan.

Refs FEAT-10 (tracker lokal; no issue di tracker eksternal)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -2424,7 +2424,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Costing / Accounting / Sales / Management</t>
+          <t>Pengguna dengan hak akses lihat</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -2434,17 +2434,17 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Filter: produk, Product Category, periode, sumber perubahan; pilihan catatan riwayat untuk melihat detail snapshot</t>
+          <t>Filter: produk, Product Category, periode, sumber perubahan; pilihan catatan riwayat untuk melihat detail snapshot; tombol Ekspor Excel</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>FR-71, NFR-17 (diusulkan; rincian diasumsikan, mohon konfirmasi OQ 34–42). 1) Setiap kali perubahan master, rate, atau input costing membuat Bottom Price suatu Produk × varian BOM berubah, sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor): waktu, pengguna yang mengubah, sumber perubahan (master/rate yang diubah, nilai lama → baru), Bottom Price lama → baru (Rp/Meter dan Rp/Kg), snapshot komponen costing lama dan baru, dan Rate Extra Margin aktif. 2) Pengguna membuka halaman History Costing. 3) Pengguna menyaring menurut produk, Product Category, periode, dan sumber perubahan. 4) Pengguna membuka detail untuk melihat snapshot komponen lama dan baru. Riwayat hanya baca (tidak dapat diubah atau dihapus), dan terpisah dari Notifikasi Bottom Price (UC-N18): notifikasi untuk Sales meninjau, riwayat untuk audit. (Permintaan user 2026-10-21.)</t>
+          <t>FR-71, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40; tafsiran terbuka OQ 43–47). 1) Setiap kali costing diperbarui dan hasilnya berubah (Bottom Price atau komponen costing suatu Produk × varian BOM berubah karena perubahan master, rate, atau input costing), sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): waktu, pengguna yang mengubah, sumber perubahan (master/rate yang diubah, nilai lama → baru), Bottom Price lama → baru (Rp/Meter dan Rp/Kg), snapshot komponen costing lama dan baru, dan Rate Extra Margin aktif. Persetujuan perubahan Rate Extra Margin oleh GM dan Draft Pricelist tidak dicatat. 2) Pengguna dengan hak akses lihat membuka halaman History Costing (menampilkan 12 bulan terakhir; riwayat lewat 1 tahun dipindahkan ke backup data, bukan dihapus). 3) Pengguna menyaring menurut produk, Product Category, periode, dan sumber perubahan. 4) Pengguna membuka detail untuk melihat snapshot komponen lama dan baru. 5) Pengguna dapat mengekspor hasil (sesuai filter) ke Excel. Riwayat hanya baca (tidak dapat diubah atau dihapus), dan terpisah dari Notifikasi Bottom Price (UC-N18): notifikasi untuk Sales meninjau, riwayat untuk audit. (Permintaan dan jawaban user 2026-10-21.)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Daftar riwayat perubahan Bottom Price dengan detail snapshot komponen lama dan baru</t>
+          <t>Daftar riwayat perubahan Bottom Price (12 bulan terakhir) dengan detail snapshot komponen lama dan baru; hasil dapat diekspor ke Excel</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Costing / Accounting / Sales / Management</t>
+          <t>Pengguna dengan hak akses lihat</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Filter: produk, Product Category, periode, kejadian; pilihan catatan riwayat untuk melihat detail</t>
+          <t>Filter: produk, Product Category, periode, kejadian; pilihan catatan riwayat untuk melihat detail; tombol Ekspor Excel</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>FR-72, NFR-17 (diusulkan; rincian diasumsikan, mohon konfirmasi OQ 34–42; terhubung ke FR-58 dan FR-67). 1) Setiap kejadian pada Pricelist disimpan per Produk × varian BOM (langkah otomatis, tanpa aktor): Diajukan, Disetujui (Approved), Ditolak (Rejected, beserta alasan), Dihitung Ulang (kembali ke Draft), atau Dirilis ke Product Catalog; dengan nomor Pricelist, status, waktu, pengguna, Price List lama → baru (Rp/Meter dan Rp/Kg), Bottom Price dan Rate Extra Margin saat itu, serta catatan atau alasan. 2) Pengguna membuka halaman History Price List. 3) Pengguna menyaring menurut produk, Product Category, periode, dan kejadian. 4) Pengguna melihat perubahan Price List lama → baru. Riwayat hanya baca (tidak dapat diubah atau dihapus). (Permintaan user 2026-10-21.)</t>
+          <t>FR-72, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40; tafsiran terbuka OQ 44–47; terhubung ke FR-58 dan FR-67). 1) Setiap kali sebuah Pricelist Disetujui (Approved) oleh Management dan menjadi harga terbaru, sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): nomor Pricelist, waktu, pengguna (penyetuju), Price List lama (Price List terakhir yang disetujui untuk produk/varian itu) → baru (Rp/Meter dan Rp/Kg), Bottom Price dan Rate Extra Margin saat itu, serta catatan. Draft, Diajukan, Ditolak, Dihitung Ulang, dan persetujuan Rate Extra Margin tidak dicatat; apakah rilis ke Product Catalog dicatat: OQ 44. 2) Pengguna dengan hak akses lihat membuka halaman History Price List (12 bulan terakhir; lewat 1 tahun dipindahkan ke backup data). 3) Pengguna menyaring menurut produk, Product Category, periode, dan kejadian. 4) Pengguna melihat perubahan Price List lama → baru. 5) Pengguna dapat mengekspor hasil (sesuai filter) ke Excel. Riwayat hanya baca (tidak dapat diubah atau dihapus). (Permintaan dan jawaban user 2026-10-21.)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Daftar riwayat kejadian Pricelist per Produk × varian BOM dengan Price List lama dan baru</t>
+          <t>Daftar riwayat Pricelist yang disetujui per Produk × varian BOM (12 bulan terakhir) dengan Price List lama dan baru; hasil dapat diekspor ke Excel</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -2574,7 +2574,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D199"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="28" customWidth="1" style="1" min="1" max="1"/>
@@ -3565,156 +3565,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3726,7 +3576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K119"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5195,7 +5045,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Menampilkan riwayat perubahan Bottom Price per Produk × varian BOM (sumber perubahan, nilai lama → baru, snapshot komponen) untuk audit; hanya baca.</t>
+          <t>Menampilkan riwayat perubahan Bottom Price per Produk × varian BOM saat costing diperbarui (sumber perubahan, nilai lama → baru, snapshot komponen) untuk audit; hanya baca; ekspor Excel.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -5205,7 +5055,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Costing, Accounting, Sales, Management: L</t>
+          <t>Pengguna dengan hak akses lihat</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -5215,7 +5065,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-71, NFR-17); rincian diasumsikan, open question 34–42. Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-71, NFR-17); OQ 34–40 terjawab 2026-10-21, tafsiran OQ 43–47. Hanya baca; menampilkan 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log); persetujuan Extra Margin tidak dicatat. Path usulan.</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -5252,7 +5102,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Menampilkan riwayat kejadian Pricelist (Diajukan, Disetujui, Ditolak, Dihitung Ulang, Dirilis) per Produk × varian BOM dengan Price List lama → baru; hanya baca.</t>
+          <t>Menampilkan riwayat Pricelist yang sudah Disetujui per Produk × varian BOM dengan Price List lama → baru; hanya baca; ekspor Excel.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -5262,7 +5112,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Costing, Accounting, Sales, Management: L</t>
+          <t>Pengguna dengan hak akses lihat</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -5272,7 +5122,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-72, NFR-17); rincian diasumsikan, open question 34–42. Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-72, NFR-17); OQ 34–40 terjawab 2026-10-21, tafsiran OQ 44–47. Hanya baca; dicatat hanya saat Disetujui (Draft dan Extra Margin tidak dicatat); 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log). Path usulan.</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -5343,36 +5193,6 @@
     <row r="87"/>
     <row r="88"/>
     <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(specs): jawaban user OQ 43-47 History (Update Costing sebagai pemicu, hak akses, backup)
- History Costing dicatat saat aksi Update Costing dijalankan dan hasil costing berbeda dari hasil
  tersimpan terakhir; rilis katalog tidak dicatat; ekspor Excel tidak memuat backup; backup diakses
  pengguna berhak; pencatatan lewat write_log (Activity Log), tabel khusus hanya bila perlu; hak akses
  View/Manage terpisah per halaman, ekspor memerlukan Manage.
- Open question baru 48 (notifikasi Bottom Price vs Update Costing) dan 49 (hak akses melihat backup).

Refs FEAT-10 (tracker lokal; no issue di tracker eksternal)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -2424,7 +2424,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Pengguna dengan hak akses lihat</t>
+          <t>Pengguna dengan hak akses View (ekspor Excel: Manage)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>FR-71, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40; tafsiran terbuka OQ 43–47). 1) Setiap kali costing diperbarui dan hasilnya berubah (Bottom Price atau komponen costing suatu Produk × varian BOM berubah karena perubahan master, rate, atau input costing), sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): waktu, pengguna yang mengubah, sumber perubahan (master/rate yang diubah, nilai lama → baru), Bottom Price lama → baru (Rp/Meter dan Rp/Kg), snapshot komponen costing lama dan baru, dan Rate Extra Margin aktif. Persetujuan perubahan Rate Extra Margin oleh GM dan Draft Pricelist tidak dicatat. 2) Pengguna dengan hak akses lihat membuka halaman History Costing (menampilkan 12 bulan terakhir; riwayat lewat 1 tahun dipindahkan ke backup data, bukan dihapus). 3) Pengguna menyaring menurut produk, Product Category, periode, dan sumber perubahan. 4) Pengguna membuka detail untuk melihat snapshot komponen lama dan baru. 5) Pengguna dapat mengekspor hasil (sesuai filter) ke Excel. Riwayat hanya baca (tidak dapat diubah atau dihapus), dan terpisah dari Notifikasi Bottom Price (UC-N18): notifikasi untuk Sales meninjau, riwayat untuk audit. (Permintaan dan jawaban user 2026-10-21.)</t>
+          <t>FR-71, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40 dan 43–47; terbuka OQ 41, 42, 48, 49). 1) Pemicu utama: aksi Update Costing (tombol di Simulasi Costing). Setiap kali Update Costing dijalankan dan hasil costing berbeda dari hasil costing terakhir yang tersimpan (Bottom Price atau komponen costing suatu Produk × varian BOM berubah karena perubahan master, rate, atau input costing), sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): waktu, pengguna yang mengubah, sumber perubahan (master/rate yang berubah sejak Update Costing sebelumnya, nilai lama → baru), Bottom Price lama → baru (Rp/Meter dan Rp/Kg), snapshot komponen costing lama dan baru, dan Rate Extra Margin aktif. Persetujuan perubahan Rate Extra Margin oleh GM dan Draft Pricelist tidak dicatat. 2) Pengguna dengan hak akses lihat membuka halaman History Costing (menampilkan 12 bulan terakhir; riwayat lewat 1 tahun dipindahkan ke backup data, bukan dihapus). 3) Pengguna menyaring menurut produk, Product Category, periode, dan sumber perubahan. 4) Pengguna membuka detail untuk melihat snapshot komponen lama dan baru. 5) Pengguna dengan hak akses Manage dapat mengekspor hasil (sesuai filter) ke Excel; ekspor tidak mencakup backup. Riwayat hanya baca (tidak dapat diubah atau dihapus), dan terpisah dari Notifikasi Bottom Price (UC-N18): notifikasi untuk Sales meninjau, riwayat untuk audit. (Permintaan dan jawaban user 2026-10-21.)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Pengguna dengan hak akses lihat</t>
+          <t>Pengguna dengan hak akses View (ekspor Excel: Manage)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -2481,12 +2481,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Filter: produk, Product Category, periode, kejadian; pilihan catatan riwayat untuk melihat detail; tombol Ekspor Excel</t>
+          <t>Filter: produk, Product Category, periode; pilihan catatan riwayat untuk melihat detail; tombol Ekspor Excel</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>FR-72, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40; tafsiran terbuka OQ 44–47; terhubung ke FR-58 dan FR-67). 1) Setiap kali sebuah Pricelist Disetujui (Approved) oleh Management dan menjadi harga terbaru, sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): nomor Pricelist, waktu, pengguna (penyetuju), Price List lama (Price List terakhir yang disetujui untuk produk/varian itu) → baru (Rp/Meter dan Rp/Kg), Bottom Price dan Rate Extra Margin saat itu, serta catatan. Draft, Diajukan, Ditolak, Dihitung Ulang, dan persetujuan Rate Extra Margin tidak dicatat; apakah rilis ke Product Catalog dicatat: OQ 44. 2) Pengguna dengan hak akses lihat membuka halaman History Price List (12 bulan terakhir; lewat 1 tahun dipindahkan ke backup data). 3) Pengguna menyaring menurut produk, Product Category, periode, dan kejadian. 4) Pengguna melihat perubahan Price List lama → baru. 5) Pengguna dapat mengekspor hasil (sesuai filter) ke Excel. Riwayat hanya baca (tidak dapat diubah atau dihapus). (Permintaan dan jawaban user 2026-10-21.)</t>
+          <t>FR-72, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40 dan 44–47; terbuka OQ 41, 42, 48, 49; terhubung ke FR-58 dan FR-67). 1) Setiap kali sebuah Pricelist Disetujui (Approved) oleh Management dan menjadi harga terbaru, sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): nomor Pricelist, waktu, pengguna (penyetuju), Price List lama (Price List terakhir yang disetujui untuk produk/varian itu) → baru (Rp/Meter dan Rp/Kg), Bottom Price dan Rate Extra Margin saat itu, serta catatan. Draft, Diajukan, Ditolak, Dihitung Ulang, dan persetujuan Rate Extra Margin tidak dicatat; rilis ke Product Catalog tidak dicatat (cukup Approval Pricelist yang menetapkan Pricelist terbaru). 2) Pengguna dengan hak akses lihat membuka halaman History Price List (12 bulan terakhir; lewat 1 tahun dipindahkan ke backup data). 3) Pengguna menyaring menurut produk, Product Category, dan periode. 4) Pengguna melihat perubahan Price List lama → baru. 5) Pengguna dengan hak akses Manage dapat mengekspor hasil (sesuai filter) ke Excel; ekspor tidak mencakup backup. Riwayat hanya baca (tidak dapat diubah atau dihapus). (Permintaan dan jawaban user 2026-10-21.)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Pengguna dengan hak akses lihat</t>
+          <t>View: lihat · Manage: ekspor Excel dan akses backup (hak akses terpisah per halaman, diatur di program; hak akses backup = tafsiran/asumsi, OQ 49)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-71, NFR-17); OQ 34–40 terjawab 2026-10-21, tafsiran OQ 43–47. Hanya baca; menampilkan 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log); persetujuan Extra Margin tidak dicatat. Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-71, NFR-17); OQ 34–40 dan 43–47 terjawab 2026-10-21; terbuka OQ 41, 42, 48, 49. Pemicu = tombol Update Costing. Ekspor Excel tidak mencakup backup. Hanya baca; menampilkan 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log); persetujuan Extra Margin tidak dicatat. Path usulan.</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Pengguna dengan hak akses lihat</t>
+          <t>View: lihat · Manage: ekspor Excel dan akses backup (hak akses terpisah per halaman, diatur di program; hak akses backup = tafsiran/asumsi, OQ 49)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-72, NFR-17); OQ 34–40 terjawab 2026-10-21, tafsiran OQ 44–47. Hanya baca; dicatat hanya saat Disetujui (Draft dan Extra Margin tidak dicatat); 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log). Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-72, NFR-17); OQ 34–40 dan 44–47 terjawab 2026-10-21; terbuka OQ 41, 42, 48, 49. Rilis katalog tidak dicatat. Ekspor Excel tidak mencakup backup. Hanya baca; dicatat hanya saat Disetujui (Draft dan Extra Margin tidak dicatat); 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log). Path usulan.</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(specs): notifikasi Bottom Price dipicu Update Costing; akses backup = Manage (OQ 48-49)
- FR-68: deteksi perubahan Bottom Price dijalankan saat Update Costing (satu pemicu dengan History
  Costing); OQ 29 direvisi. NFR-17/FR-71/FR-72: akses data backup = hak Manage.
- UC-N18 dan UC-N19/N20, PG-24..26, vocabulary (Update Costing), intake dan log disesuaikan.

Refs FEAT-09, FEAT-10 (tracker lokal; no issue di tracker eksternal)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -2392,7 +2392,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>FR-68, FR-69, FR-70, NFR-16 (diusulkan; seluruh rincian dikonfirmasi user 2026-10-21 — OQ 25–33). 1) Sistem membandingkan Bottom Price (Rp/Meter dan Rp/Kg) tiap Produk × varian BOM dengan baseline setiap kali costing dihitung; bila berbeda (naik atau turun, apa pun penyebabnya) sistem membuat notifikasi berstatus Belum Ditinjau (langkah otomatis, tanpa aktor). 2) Sales (Staf Sales atau Sales Manager) membuka dashboard notifikasi; notifikasi dikelompokkan per Product Category dan jumlah yang belum ditinjau tampil sebagai lencana di menu. 3) Sales membandingkan Bottom Price lama dan baru, selisih (Rp dan %), komponen yang berubah, Rate Extra Margin aktif, harga jual saat ini terhadap Price List baru bila rate lama dipertahankan. 4) Sales memilih: a) Ajukan Rate Extra Margin Baru (hanya Sales Manager; hak akses diatur per pengguna di program): membuka pengajuan UC-12 untuk Product Category itu, lalu GM memutuskan di UC-16 (FR-67); status Diajukan Extra Margin Baru dan terhubung ke pengajuan; b) Tidak Perlu Diubah (catatan opsional): status Tidak Perlu Diubah. 5) Kedua keputusan mencatat peninjau, waktu, dan catatan, ditulis ke log, dan menggeser baseline ke Bottom Price baru. Sistem tidak mengubah rate, Pricelist, atau Katalog secara otomatis. Semua Sales dapat meninjau; kanal hanya dashboard (tanpa email/WhatsApp) dan tanpa batas waktu tinjau; ambang: perubahan sekecil apa pun (≥ Rp0,01). Di luar scope: persetujuan diskon Quotation. (Permintaan user 2026-10-21; terkait BPMN To Be Sales D01, gateway "Perlu Perubahan Margin?".)</t>
+          <t>FR-68, FR-69, FR-70, NFR-16 (diusulkan; seluruh rincian dikonfirmasi user 2026-10-21 — OQ 25–33 dan 48). 1) Sistem membandingkan Bottom Price (Rp/Meter dan Rp/Kg) tiap Produk × varian BOM dengan baseline setiap kali Update Costing dijalankan (tombol di Simulasi Costing, oleh pengguna yang menjalankan Update Costing; pemicu yang sama dengan History Costing, OQ 48); bila berbeda (naik atau turun, apa pun penyebabnya) sistem membuat notifikasi berstatus Belum Ditinjau (langkah otomatis setelah Update Costing). 2) Sales (Staf Sales atau Sales Manager) membuka dashboard notifikasi; notifikasi dikelompokkan per Product Category dan jumlah yang belum ditinjau tampil sebagai lencana di menu. 3) Sales membandingkan Bottom Price lama dan baru, selisih (Rp dan %), komponen yang berubah, Rate Extra Margin aktif, harga jual saat ini terhadap Price List baru bila rate lama dipertahankan. 4) Sales memilih: a) Ajukan Rate Extra Margin Baru (hanya Sales Manager; hak akses diatur per pengguna di program): membuka pengajuan UC-12 untuk Product Category itu, lalu GM memutuskan di UC-16 (FR-67); status Diajukan Extra Margin Baru dan terhubung ke pengajuan; b) Tidak Perlu Diubah (catatan opsional): status Tidak Perlu Diubah. 5) Kedua keputusan mencatat peninjau, waktu, dan catatan, ditulis ke log, dan menggeser baseline ke Bottom Price baru. Sistem tidak mengubah rate, Pricelist, atau Katalog secara otomatis. Semua Sales dapat meninjau; kanal hanya dashboard (tanpa email/WhatsApp) dan tanpa batas waktu tinjau; ambang: perubahan sekecil apa pun (≥ Rp0,01). Di luar scope: persetujuan diskon Quotation. (Permintaan user 2026-10-21; terkait BPMN To Be Sales D01, gateway "Perlu Perubahan Margin?".)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>FR-71, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40 dan 43–47; terbuka OQ 41, 42, 48, 49). 1) Pemicu utama: aksi Update Costing (tombol di Simulasi Costing). Setiap kali Update Costing dijalankan dan hasil costing berbeda dari hasil costing terakhir yang tersimpan (Bottom Price atau komponen costing suatu Produk × varian BOM berubah karena perubahan master, rate, atau input costing), sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): waktu, pengguna yang mengubah, sumber perubahan (master/rate yang berubah sejak Update Costing sebelumnya, nilai lama → baru), Bottom Price lama → baru (Rp/Meter dan Rp/Kg), snapshot komponen costing lama dan baru, dan Rate Extra Margin aktif. Persetujuan perubahan Rate Extra Margin oleh GM dan Draft Pricelist tidak dicatat. 2) Pengguna dengan hak akses lihat membuka halaman History Costing (menampilkan 12 bulan terakhir; riwayat lewat 1 tahun dipindahkan ke backup data, bukan dihapus). 3) Pengguna menyaring menurut produk, Product Category, periode, dan sumber perubahan. 4) Pengguna membuka detail untuk melihat snapshot komponen lama dan baru. 5) Pengguna dengan hak akses Manage dapat mengekspor hasil (sesuai filter) ke Excel; ekspor tidak mencakup backup. Riwayat hanya baca (tidak dapat diubah atau dihapus), dan terpisah dari Notifikasi Bottom Price (UC-N18): notifikasi untuk Sales meninjau, riwayat untuk audit. (Permintaan dan jawaban user 2026-10-21.)</t>
+          <t>FR-71, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40 dan 43–49; terbuka OQ 41, 42). 1) Pemicu utama: aksi Update Costing (tombol di Simulasi Costing). Setiap kali Update Costing dijalankan dan hasil costing berbeda dari hasil costing terakhir yang tersimpan (Bottom Price atau komponen costing suatu Produk × varian BOM berubah karena perubahan master, rate, atau input costing), sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): waktu, pengguna yang mengubah, sumber perubahan (master/rate yang berubah sejak Update Costing sebelumnya, nilai lama → baru), Bottom Price lama → baru (Rp/Meter dan Rp/Kg), snapshot komponen costing lama dan baru, dan Rate Extra Margin aktif. Persetujuan perubahan Rate Extra Margin oleh GM dan Draft Pricelist tidak dicatat. 2) Pengguna dengan hak akses lihat membuka halaman History Costing (menampilkan 12 bulan terakhir; riwayat lewat 1 tahun dipindahkan ke backup data, bukan dihapus). 3) Pengguna menyaring menurut produk, Product Category, periode, dan sumber perubahan. 4) Pengguna membuka detail untuk melihat snapshot komponen lama dan baru. 5) Pengguna dengan hak akses Manage dapat mengekspor hasil (sesuai filter) ke Excel; ekspor tidak mencakup backup. Riwayat hanya baca (tidak dapat diubah atau dihapus), dan terpisah dari Notifikasi Bottom Price (UC-N18): notifikasi untuk Sales meninjau, riwayat untuk audit. (Permintaan dan jawaban user 2026-10-21.)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>FR-72, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40 dan 44–47; terbuka OQ 41, 42, 48, 49; terhubung ke FR-58 dan FR-67). 1) Setiap kali sebuah Pricelist Disetujui (Approved) oleh Management dan menjadi harga terbaru, sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): nomor Pricelist, waktu, pengguna (penyetuju), Price List lama (Price List terakhir yang disetujui untuk produk/varian itu) → baru (Rp/Meter dan Rp/Kg), Bottom Price dan Rate Extra Margin saat itu, serta catatan. Draft, Diajukan, Ditolak, Dihitung Ulang, dan persetujuan Rate Extra Margin tidak dicatat; rilis ke Product Catalog tidak dicatat (cukup Approval Pricelist yang menetapkan Pricelist terbaru). 2) Pengguna dengan hak akses lihat membuka halaman History Price List (12 bulan terakhir; lewat 1 tahun dipindahkan ke backup data). 3) Pengguna menyaring menurut produk, Product Category, dan periode. 4) Pengguna melihat perubahan Price List lama → baru. 5) Pengguna dengan hak akses Manage dapat mengekspor hasil (sesuai filter) ke Excel; ekspor tidak mencakup backup. Riwayat hanya baca (tidak dapat diubah atau dihapus). (Permintaan dan jawaban user 2026-10-21.)</t>
+          <t>FR-72, NFR-17 (dikonfirmasi user 2026-10-21, OQ 34–40 dan 44–49; terbuka OQ 41, 42; terhubung ke FR-58 dan FR-67). 1) Setiap kali sebuah Pricelist Disetujui (Approved) oleh Management dan menjadi harga terbaru, sistem menyimpan satu catatan riwayat per Produk × varian BOM (langkah otomatis, tanpa aktor, lewat write_log() sehingga juga tampil di Activity Log): nomor Pricelist, waktu, pengguna (penyetuju), Price List lama (Price List terakhir yang disetujui untuk produk/varian itu) → baru (Rp/Meter dan Rp/Kg), Bottom Price dan Rate Extra Margin saat itu, serta catatan. Draft, Diajukan, Ditolak, Dihitung Ulang, dan persetujuan Rate Extra Margin tidak dicatat; rilis ke Product Catalog tidak dicatat (cukup Approval Pricelist yang menetapkan Pricelist terbaru). 2) Pengguna dengan hak akses lihat membuka halaman History Price List (12 bulan terakhir; lewat 1 tahun dipindahkan ke backup data). 3) Pengguna menyaring menurut produk, Product Category, dan periode. 4) Pengguna melihat perubahan Price List lama → baru. 5) Pengguna dengan hak akses Manage dapat mengekspor hasil (sesuai filter) ke Excel; ekspor tidak mencakup backup. Riwayat hanya baca (tidak dapat diubah atau dihapus). (Permintaan dan jawaban user 2026-10-21.)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist; lencana jumlah notifikasi Belum Ditinjau di menu. Fitur diusulkan (FR-68–FR-70, NFR-16); rincian diasumsikan, open question 25–33 terjawab 2026-10-21. Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist; lencana jumlah notifikasi Belum Ditinjau di menu. Fitur diusulkan (FR-68–FR-70, NFR-16); rincian diasumsikan, open question 25–33 dan 48 terjawab 2026-10-21 (pemicu deteksi = Update Costing). Path usulan.</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>View: lihat · Manage: ekspor Excel dan akses backup (hak akses terpisah per halaman, diatur di program; hak akses backup = tafsiran/asumsi, OQ 49)</t>
+          <t>View: lihat · Manage: ekspor Excel dan akses backup (hak akses terpisah per halaman, diatur di program; hak akses backup = Manage, dikonfirmasi user 2026-10-21, OQ 49)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-71, NFR-17); OQ 34–40 dan 43–47 terjawab 2026-10-21; terbuka OQ 41, 42, 48, 49. Pemicu = tombol Update Costing. Ekspor Excel tidak mencakup backup. Hanya baca; menampilkan 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log); persetujuan Extra Margin tidak dicatat. Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-71, NFR-17); OQ 34–40 dan 43–47 terjawab 2026-10-21; terbuka OQ 41, 42; OQ 48 dan 49 terjawab 2026-10-21. Pemicu = tombol Update Costing. Ekspor Excel tidak mencakup backup. Hanya baca; menampilkan 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log); persetujuan Extra Margin tidak dicatat. Path usulan.</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>View: lihat · Manage: ekspor Excel dan akses backup (hak akses terpisah per halaman, diatur di program; hak akses backup = tafsiran/asumsi, OQ 49)</t>
+          <t>View: lihat · Manage: ekspor Excel dan akses backup (hak akses terpisah per halaman, diatur di program; hak akses backup = Manage, dikonfirmasi user 2026-10-21, OQ 49)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-72, NFR-17); OQ 34–40 dan 44–47 terjawab 2026-10-21; terbuka OQ 41, 42, 48, 49. Rilis katalog tidak dicatat. Ekspor Excel tidak mencakup backup. Hanya baca; dicatat hanya saat Disetujui (Draft dan Extra Margin tidak dicatat); 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log). Path usulan.</t>
+          <t>menu Hasil &amp; Pricelist. Fitur diusulkan (FR-72, NFR-17); OQ 34–40 dan 44–47 terjawab 2026-10-21; terbuka OQ 41, 42; OQ 48 dan 49 terjawab 2026-10-21. Rilis katalog tidak dicatat. Ekspor Excel tidak mencakup backup. Hanya baca; dicatat hanya saat Disetujui (Draft dan Extra Margin tidak dicatat); 12 bulan terakhir (lebih lama di backup data); pencatatan lewat write_log (Activity Log). Path usulan.</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: HPP komponen memakai Rp/Kg Hasil Costing varian BOM; Add SPK pilih varian (FR-48, FR-74)
Refs FEAT-08

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -799,7 +799,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi).</t>
+          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi). [2026-10-26, FR-48 direvisi/FR-74] Saat Add SPK, setelah memilih produk, pengguna memilih varian BOM (uniq_id); dibawa ke item laporan (OQ 50-55).</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -1236,7 +1236,7 @@
       <c r="F12" s="3" t="inlineStr">
         <is>
           <t>FR-24: Accounting melakukan Posting Jurnal Produksi ke GL Interface berdasarkan Nilai Material dan HPP hasil FR-19 s.d. FR-23, mencakup jurnal: KW1, KW2, Scrap, Inventory, Hutang Biaya Proses, Hutang Scrap, dan Hutang Koordinasi.
-Field-level dari ERD revisi klien (Rev.2, menggantikan Rev.1), bukan UC terpisah: FR-34 - komponen biaya HPP per item (tujuh komponen x *_cost_per_pcs/*_cost_total, plus total_hpp_item) pada production_report_items, dibedakan oleh category_type; menggantikan FR-28. FR-35 - scrap per baris (scrap_type, qty, berat_total, berat_material_plat) pada production_report_scraps; menggantikan FR-27. Total HPP keseluruhan pada header production_reports (total_hpp_keseluruhan, FR-32). Catatan: pemisahan 80%/20% (KW 2) dan 40%/60% (scrap) belum punya kolom di Rev.2 (open question, belum dikonfirmasi).</t>
+Field-level dari ERD revisi klien (Rev.2, menggantikan Rev.1), bukan UC terpisah: FR-34 - komponen biaya HPP per item (tujuh komponen x *_cost_per_pcs/*_cost_total, plus total_hpp_item) pada production_report_items, dibedakan oleh category_type; menggantikan FR-28. FR-35 - scrap per baris (scrap_type, qty, berat_total, berat_material_plat) pada production_report_scraps; menggantikan FR-27. Total HPP keseluruhan pada header production_reports (total_hpp_keseluruhan, FR-32). Catatan: pemisahan 80%/20% (KW 2) dan 40%/60% (scrap) belum punya kolom di Rev.2 (open question, belum dikonfirmasi). [2026-10-26, FR-48 direvisi/FR-74] Komponen HPP selain Material = Rp/Kg Hasil Costing varian BOM x berat per pcs (bukan Master Rate rate.html).</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -2505,64 +2505,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3576,7 +3518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3868,7 +3810,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view).</t>
+          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view). [2026-10-26, FR-48 direvisi/FR-74] Add SPK: pilih varian BOM setelah produk.</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -3925,7 +3867,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>menu Produksi (HPP). Modul gl_interface sudah ada (index, data, detail, view, post, post_batch).</t>
+          <t>menu Produksi (HPP). Modul gl_interface sudah ada (index, data, detail, view, post, post_batch). [2026-10-26, FR-48 direvisi/FR-74] Rate komponen biaya dari Hasil Costing (pc-simulasi) varian BOM SPK; rate.html tidak lagi dipakai.</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -5131,68 +5073,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(mockup): HPP memakai Rp/Kg Hasil Costing per varian BOM; Add SPK pilih varian, tolak tanpa costing; rate.html dipensiunkan; OQ 50-55 selesai (FEAT-08)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -799,7 +799,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi). [2026-10-26, FR-48 direvisi/FR-74] Saat Add SPK, setelah memilih produk, pengguna memilih varian BOM (uniq_id); dibawa ke item laporan (OQ 50-55).</t>
+          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi). [2026-10-26, FR-48 direvisi/FR-74] Saat Add SPK, setelah memilih produk, pengguna memilih varian BOM (uniq_id); dibawa ke item laporan (OQ 50-55). [2026-10-26, OQ 50/51/53/55 dijawab] SPK ditolak bila produk tanpa varian BOM atau Hasil Costing belum lengkap; varian per produk; varian dapat diubah selama SPK belum diinput laporan produksinya; SPK dibuat di modul Production Planning (eksternal).</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view). [2026-10-26, FR-48 direvisi/FR-74] Add SPK: pilih varian BOM setelah produk.</t>
+          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view). [2026-10-26, FR-48 direvisi/FR-74] Add SPK: pilih varian BOM setelah produk. [2026-10-26, OQ 50/51/53/55] SPK ditolak bila produk tanpa varian BOM/Hasil Costing lengkap; varian per produk; terkunci setelah laporan produksi diinput; Add SPK di mockup hanya simulasi modul Production Planning (eksternal).</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>menu Produksi (HPP). Modul gl_interface sudah ada (index, data, detail, view, post, post_batch). [2026-10-26, FR-48 direvisi/FR-74] Rate komponen biaya dari Hasil Costing (pc-simulasi) varian BOM SPK; rate.html tidak lagi dipakai.</t>
+          <t>menu Produksi (HPP). Modul gl_interface sudah ada (index, data, detail, view, post, post_batch). [2026-10-26, FR-48 direvisi/FR-74] Rate komponen biaya dari Hasil Costing (pc-simulasi) varian BOM SPK; rate.html (Master Rate lama) dipensiunkan (OQ 54, dijawab user 2026-10-26).</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: varian_type di ERD resmi erd-revisi.drawio dan label tampilan Varian BOM (varian_type) (FEAT-08)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -799,7 +799,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi). [2026-10-26, FR-48 direvisi/FR-74] Saat Add SPK, setelah memilih produk, pengguna memilih varian BOM (uniq_id); dibawa ke item laporan (OQ 50-55). [2026-10-26, OQ 50/51/53/55 dijawab] SPK ditolak bila produk tanpa varian BOM atau Hasil Costing belum lengkap; varian per produk; varian dapat diubah selama SPK belum diinput laporan produksinya; SPK dibuat di modul Production Planning (eksternal).</t>
+          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi). [2026-10-26, FR-48 direvisi/FR-74] Saat Add SPK, setelah memilih produk, pengguna memilih varian BOM (kolom varian_type; label tampilan Varian BOM (varian_type)); dibawa ke item laporan (OQ 50-55). [2026-10-26, OQ 50/51/53/55 dijawab] SPK ditolak bila produk tanpa varian BOM atau Hasil Costing belum lengkap; varian per produk; varian dapat diubah selama SPK belum diinput laporan produksinya; SPK dibuat di modul Production Planning (eksternal). [2026-10-26, varian_type] Item Stok Bebas dan KW 2 pada laporan produksi mengikuti varian BOM yang dipilih di SPK; ERD yang diperbarui = erd-revisi.drawio.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view). [2026-10-26, FR-48 direvisi/FR-74] Add SPK: pilih varian BOM setelah produk. [2026-10-26, OQ 50/51/53/55] SPK ditolak bila produk tanpa varian BOM/Hasil Costing lengkap; varian per produk; terkunci setelah laporan produksi diinput; Add SPK di mockup hanya simulasi modul Production Planning (eksternal).</t>
+          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view). [2026-10-26, FR-48 direvisi/FR-74] Add SPK: pilih varian BOM setelah produk (kolom varian_type; label Varian BOM (varian_type)). [2026-10-26, OQ 50/51/53/55] SPK ditolak bila produk tanpa varian BOM/Hasil Costing lengkap; varian per produk; terkunci setelah laporan produksi diinput; Add SPK di mockup hanya simulasi modul Production Planning (eksternal).</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: BOM Product Costing memakai ms_bom_header dan ms_bom_detail (FEAT-04)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -1969,7 +1969,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>FR-41, FR-51. Prasyarat: Master Produk (UC-N05), Master Material (UC-N06), Master Standard Material (UC-N15). 1) Engineering membuka daftar BOM per produk. 2) Engineering menambah varian BOM (Varian Tebal) untuk produk dengan memilih material dari Master Material. 3) Sistem menghitung Berat/Meter (kg/m) = ((Tebal Material − Standar Toleransi) × Lebar Coil × Standar Berat Jenis) + Coating dari Master Standard Material (global; satuan tidak ditampilkan, konversi dikalibrasi 0,14 mm × lebar 1219 × 7,85 ≈ 1,34 kg/m — FR-50) dan menyimpannya pada bom_detail. 4) Sistem membuat No. Uniq ID per varian (mis. Type 001.1) dan mengisi Latest Update dan Updated By. 5) Engineering dapat View, Edit, atau Delete varian. Satu produk boleh memakai beberapa material, tetapi tidak boleh memakai material yang sama dua kali (unik produk + material). (Rev.1 UC-04; BPMN D05: 'Develop BOM Produk berdasarkan Varian Tebal'.)</t>
+          <t>FR-41, FR-51. Prasyarat: Master Produk (UC-N05), Master Material (UC-N06), Master Standard Material (UC-N15). 1) Engineering membuka daftar BOM per produk. 2) Engineering menambah varian BOM (Varian Tebal) untuk produk dengan memilih material dari Master Material. 3) Sistem menghitung Berat/Meter (kg/m) = ((Tebal Material − Standar Toleransi) × Lebar Coil × Standar Berat Jenis) + Coating dari Master Standard Material (global; satuan tidak ditampilkan, konversi dikalibrasi 0,14 mm × lebar 1219 × 7,85 ≈ 1,34 kg/m — FR-50) dan menyimpannya pada ms_bom_detail. 4) Sistem membuat No. Uniq ID per varian (mis. Type 001.1) dan mengisi Latest Update dan Updated By. 5) Engineering dapat View, Edit, atau Delete varian. Satu produk boleh memakai beberapa material, tetapi tidak boleh memakai material yang sama dua kali (unik produk + material). (Rev.1 UC-04; BPMN D05: 'Develop BOM Produk berdasarkan Varian Tebal'.)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>bom_header, bom_detail, product_lvl_4, material, master_standard_material</t>
+          <t>ms_bom_header, ms_bom_detail, product_lvl_4, material, master_standard_material</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>product_costing_header, product_costing_detail, material_cost, man_power_cost, bom_header, bom_detail, price_reference_header, price_reference_detail, flow_process_header, man_power_rate, rate_borongan_helper, rate_bahan_pendukung_foh, rate_generals, master_kurs, product_lvl_4</t>
+          <t>product_costing_header, product_costing_detail, material_cost, man_power_cost, ms_bom_header, ms_bom_detail, price_reference_header, price_reference_detail, flow_process_header, man_power_rate, rate_borongan_helper, rate_bahan_pendukung_foh, rate_generals, master_kurs, product_lvl_4</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -3150,7 +3150,7 @@
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>bom_header</t>
+          <t>ms_bom_header</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3170,7 +3170,7 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>bom_detail</t>
+          <t>ms_bom_detail</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: identitas varian BOM = ms_bom_detail.no_uniq_id (menggantikan varian_type); label Varian BOM (no_uniq_id) (FEAT-04, FEAT-08)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/specs/docs/workbook.xlsx
+++ b/specs/docs/workbook.xlsx
@@ -799,7 +799,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi). [2026-10-26, FR-48 direvisi/FR-74] Saat Add SPK, setelah memilih produk, pengguna memilih varian BOM (kolom varian_type; label tampilan Varian BOM (varian_type)); dibawa ke item laporan (OQ 50-55). [2026-10-26, OQ 50/51/53/55 dijawab] SPK ditolak bila produk tanpa varian BOM atau Hasil Costing belum lengkap; varian per produk; varian dapat diubah selama SPK belum diinput laporan produksinya; SPK dibuat di modul Production Planning (eksternal). [2026-10-26, varian_type] Item Stok Bebas dan KW 2 pada laporan produksi mengikuti varian BOM yang dipilih di SPK; ERD yang diperbarui = erd-revisi.drawio.</t>
+          <t>FR-05 dan FR-06 (bagian Operator): Setelah unpacking, Operator melakukan Cek Kondisi Coil — pemeriksaan fisik (Manual task, dikecualikan dari UC, tanpa keterlibatan sistem). Bila hasilnya 'Tidak sesuai', Operator menginput Laporan Ketidaksesuaian Material ke sistem, yang kemudian dikirim ke Claim Material (proses lain, di luar Modul Produksi). [2026-10-26, FR-48 direvisi/FR-74] Saat Add SPK, setelah memilih produk, pengguna memilih varian BOM (kolom no_uniq_id; label tampilan Varian BOM (no_uniq_id)); dibawa ke item laporan (OQ 50-55). [2026-10-26, OQ 50/51/53/55 dijawab] SPK ditolak bila produk tanpa varian BOM atau Hasil Costing belum lengkap; varian per produk; varian dapat diubah selama SPK belum diinput laporan produksinya; SPK dibuat di modul Production Planning (eksternal). [2026-10-26, no_uniq_id] Item Stok Bebas dan KW 2 pada laporan produksi mengikuti varian BOM yang dipilih di SPK; ERD yang diperbarui = erd-revisi.drawio. [2026-10-26, direvisi] Kolom varian = ms_bom_detail.no_uniq_id (menggantikan varian_type; kunci pasangan id_produk + no_uniq_id).</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>FR-41, FR-51. Prasyarat: Master Produk (UC-N05), Master Material (UC-N06), Master Standard Material (UC-N15). 1) Engineering membuka daftar BOM per produk. 2) Engineering menambah varian BOM (Varian Tebal) untuk produk dengan memilih material dari Master Material. 3) Sistem menghitung Berat/Meter (kg/m) = ((Tebal Material − Standar Toleransi) × Lebar Coil × Standar Berat Jenis) + Coating dari Master Standard Material (global; satuan tidak ditampilkan, konversi dikalibrasi 0,14 mm × lebar 1219 × 7,85 ≈ 1,34 kg/m — FR-50) dan menyimpannya pada ms_bom_detail. 4) Sistem membuat No. Uniq ID per varian (mis. Type 001.1) dan mengisi Latest Update dan Updated By. 5) Engineering dapat View, Edit, atau Delete varian. Satu produk boleh memakai beberapa material, tetapi tidak boleh memakai material yang sama dua kali (unik produk + material). (Rev.1 UC-04; BPMN D05: 'Develop BOM Produk berdasarkan Varian Tebal'.)</t>
+          <t>FR-41, FR-51. Prasyarat: Master Produk (UC-N05), Master Material (UC-N06), Master Standard Material (UC-N15). 1) Engineering membuka daftar BOM per produk. 2) Engineering menambah varian BOM (Varian Tebal) untuk produk dengan memilih material dari Master Material. 3) Sistem menghitung Berat/Meter (kg/m) = ((Tebal Material − Standar Toleransi) × Lebar Coil × Standar Berat Jenis) + Coating dari Master Standard Material (global; satuan tidak ditampilkan, konversi dikalibrasi 0,14 mm × lebar 1219 × 7,85 ≈ 1,34 kg/m — FR-50) dan menyimpannya pada ms_bom_detail. 4) Sistem membuat No. Uniq ID per varian (mis. Type 001.1) dan mengisi Latest Update dan Updated By. 5) Engineering dapat View, Edit, atau Delete varian. Satu produk boleh memakai beberapa material, tetapi tidak boleh memakai material yang sama dua kali (unik produk + material). (Rev.1 UC-04; BPMN D05: 'Develop BOM Produk berdasarkan Varian Tebal'.) [2026-10-26, definisi varian] Satu varian = satu baris material pada BOM produk (ms_bom_detail); produk dengan beberapa material berbeda ketebalan punya beberapa varian; satu header ms_bom_header per produk (UNIQUE id_produk tetap); kunci varian = pasangan id_produk + no_uniq_id; ms_bom_header.varian_type dan is_default hanya kompatibilitas.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view). [2026-10-26, FR-48 direvisi/FR-74] Add SPK: pilih varian BOM setelah produk (kolom varian_type; label Varian BOM (varian_type)). [2026-10-26, OQ 50/51/53/55] SPK ditolak bila produk tanpa varian BOM/Hasil Costing lengkap; varian per produk; terkunci setelah laporan produksi diinput; Add SPK di mockup hanya simulasi modul Production Planning (eksternal).</t>
+          <t>menu Produksi (Daftar SPK, Input Produksi). Satu aktor, satu sitting, satu entitas (production_reports); 11 UC dalam satu halaman bersektor. Modul sudah ada (index, ajax_spk_list, create, ajax_get_coils, save, view). [2026-10-26, FR-48 direvisi/FR-74] Add SPK: pilih varian BOM setelah produk (kolom no_uniq_id; label Varian BOM (no_uniq_id)). [2026-10-26, OQ 50/51/53/55] SPK ditolak bila produk tanpa varian BOM/Hasil Costing lengkap; varian per produk; terkunci setelah laporan produksi diinput; Add SPK di mockup hanya simulasi modul Production Planning (eksternal). [2026-10-26, direvisi] Kolom varian = ms_bom_detail.no_uniq_id (menggantikan varian_type; kunci pasangan id_produk + no_uniq_id).</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">

</xml_diff>